<commit_message>
Enhance chronological barcode reconciliation: auto-overwrite valid barcodes from subsequent dates and preserve existing barcodes
</commit_message>
<xml_diff>
--- a/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
+++ b/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
@@ -152,7 +152,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="9">
     <border>
       <left/>
       <right/>
@@ -188,11 +188,75 @@
         <color rgb="001D1D1B"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="001D1D1B"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="medium">
+        <color rgb="001D1D1B"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color rgb="001D1D1B"/>
+      </top>
+      <bottom style="double">
+        <color rgb="001D1D1B"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top style="medium">
+        <color rgb="001D1D1B"/>
+      </top>
+      <bottom style="double">
+        <color rgb="001D1D1B"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top/>
+      <bottom style="double">
+        <color rgb="001D1D1B"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CBD5E1"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="36">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center"/>
@@ -285,6 +349,12 @@
     <xf numFmtId="0" fontId="3" fillId="9" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="7" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -677,7 +747,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -9438,12 +9507,12 @@
       </c>
       <c r="D249" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>34330</t>
         </is>
       </c>
       <c r="E249" s="4" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>52</t>
         </is>
       </c>
       <c r="F249" s="14" t="n">
@@ -9451,14 +9520,10 @@
       </c>
       <c r="G249" s="7" t="inlineStr">
         <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="H249" s="8" t="inlineStr">
-        <is>
-          <t>out</t>
-        </is>
-      </c>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H249" s="8" t="inlineStr"/>
     </row>
     <row r="250" ht="20" customHeight="1">
       <c r="A250" s="9" t="n">
@@ -9474,27 +9539,23 @@
       </c>
       <c r="D250" s="9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>34329</t>
         </is>
       </c>
       <c r="E250" s="9" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>52</t>
         </is>
       </c>
       <c r="F250" s="17" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="G250" s="7" t="inlineStr">
         <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="H250" s="12" t="inlineStr">
-        <is>
-          <t>out mabe</t>
-        </is>
-      </c>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H250" s="12" t="inlineStr"/>
     </row>
     <row r="251" ht="20" customHeight="1">
       <c r="A251" s="4" t="n">
@@ -13364,11 +13425,7 @@
           <t>SELESAI</t>
         </is>
       </c>
-      <c r="H358" s="12" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="H358" s="12" t="inlineStr"/>
     </row>
     <row r="359" ht="20" customHeight="1">
       <c r="A359" s="4" t="n">
@@ -13400,11 +13457,7 @@
           <t>SELESAI</t>
         </is>
       </c>
-      <c r="H359" s="8" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
+      <c r="H359" s="8" t="inlineStr"/>
     </row>
     <row r="360" ht="20" customHeight="1">
       <c r="A360" s="9" t="n">
@@ -17116,10 +17169,10 @@
           <t>TOTAL KESELURUHAN</t>
         </is>
       </c>
-      <c r="B463" s="21" t="n"/>
-      <c r="C463" s="21" t="n"/>
-      <c r="D463" s="21" t="n"/>
-      <c r="E463" s="21" t="n"/>
+      <c r="B463" s="32" t="n"/>
+      <c r="C463" s="32" t="n"/>
+      <c r="D463" s="32" t="n"/>
+      <c r="E463" s="33" t="n"/>
       <c r="F463" s="22">
         <f>SUM(F5:F462)</f>
         <v/>
@@ -17172,7 +17225,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -18828,9 +18880,9 @@
           <t>TOTAL HARI INI</t>
         </is>
       </c>
-      <c r="B57" s="21" t="n"/>
-      <c r="C57" s="21" t="n"/>
-      <c r="D57" s="21" t="n"/>
+      <c r="B57" s="32" t="n"/>
+      <c r="C57" s="32" t="n"/>
+      <c r="D57" s="33" t="n"/>
       <c r="E57" s="22">
         <f>SUM(E5:E56)</f>
         <v/>
@@ -18883,7 +18935,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -19574,9 +19625,9 @@
           <t>TOTAL HARI INI</t>
         </is>
       </c>
-      <c r="B26" s="21" t="n"/>
-      <c r="C26" s="21" t="n"/>
-      <c r="D26" s="21" t="n"/>
+      <c r="B26" s="32" t="n"/>
+      <c r="C26" s="32" t="n"/>
+      <c r="D26" s="33" t="n"/>
       <c r="E26" s="22">
         <f>SUM(E5:E25)</f>
         <v/>
@@ -19629,7 +19680,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="3" t="inlineStr">
         <is>
@@ -19893,12 +19943,12 @@
       </c>
     </row>
     <row r="14" ht="24" customHeight="1">
-      <c r="A14" s="30" t="inlineStr">
+      <c r="A14" s="34" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B14" s="21" t="n"/>
+      <c r="B14" s="35" t="n"/>
       <c r="C14" s="23">
         <f>SUM(C5:C13)</f>
         <v/>
@@ -19962,7 +20012,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -21891,9 +21940,9 @@
           <t>TOTAL HARI INI</t>
         </is>
       </c>
-      <c r="B66" s="21" t="n"/>
-      <c r="C66" s="21" t="n"/>
-      <c r="D66" s="21" t="n"/>
+      <c r="B66" s="32" t="n"/>
+      <c r="C66" s="32" t="n"/>
+      <c r="D66" s="33" t="n"/>
       <c r="E66" s="22">
         <f>SUM(E5:E65)</f>
         <v/>
@@ -21946,7 +21995,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -23875,9 +23923,9 @@
           <t>TOTAL HARI INI</t>
         </is>
       </c>
-      <c r="B66" s="21" t="n"/>
-      <c r="C66" s="21" t="n"/>
-      <c r="D66" s="21" t="n"/>
+      <c r="B66" s="32" t="n"/>
+      <c r="C66" s="32" t="n"/>
+      <c r="D66" s="33" t="n"/>
       <c r="E66" s="22">
         <f>SUM(E5:E65)</f>
         <v/>
@@ -23930,7 +23978,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -25756,9 +25803,9 @@
           <t>TOTAL HARI INI</t>
         </is>
       </c>
-      <c r="B63" s="21" t="n"/>
-      <c r="C63" s="21" t="n"/>
-      <c r="D63" s="21" t="n"/>
+      <c r="B63" s="32" t="n"/>
+      <c r="C63" s="32" t="n"/>
+      <c r="D63" s="33" t="n"/>
       <c r="E63" s="22">
         <f>SUM(E5:E62)</f>
         <v/>
@@ -25811,7 +25858,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -27303,9 +27349,9 @@
           <t>TOTAL HARI INI</t>
         </is>
       </c>
-      <c r="B53" s="21" t="n"/>
-      <c r="C53" s="21" t="n"/>
-      <c r="D53" s="21" t="n"/>
+      <c r="B53" s="32" t="n"/>
+      <c r="C53" s="32" t="n"/>
+      <c r="D53" s="33" t="n"/>
       <c r="E53" s="22">
         <f>SUM(E5:E52)</f>
         <v/>
@@ -27358,7 +27404,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -27889,12 +27934,12 @@
       </c>
       <c r="C21" s="4" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>34330</t>
         </is>
       </c>
       <c r="D21" s="4" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>52</t>
         </is>
       </c>
       <c r="E21" s="14" t="n">
@@ -27902,14 +27947,10 @@
       </c>
       <c r="F21" s="7" t="inlineStr">
         <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="G21" s="8" t="inlineStr">
-        <is>
-          <t>out</t>
-        </is>
-      </c>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G21" s="8" t="inlineStr"/>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="9" t="n">
@@ -27920,27 +27961,23 @@
       </c>
       <c r="C22" s="9" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>34329</t>
         </is>
       </c>
       <c r="D22" s="9" t="inlineStr">
         <is>
-          <t>66</t>
+          <t>52</t>
         </is>
       </c>
       <c r="E22" s="17" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="F22" s="7" t="inlineStr">
         <is>
-          <t>OUT</t>
-        </is>
-      </c>
-      <c r="G22" s="12" t="inlineStr">
-        <is>
-          <t>out mabe</t>
-        </is>
-      </c>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G22" s="12" t="inlineStr"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="4" t="n">
@@ -29393,9 +29430,9 @@
           <t>TOTAL HARI INI</t>
         </is>
       </c>
-      <c r="B70" s="21" t="n"/>
-      <c r="C70" s="21" t="n"/>
-      <c r="D70" s="21" t="n"/>
+      <c r="B70" s="32" t="n"/>
+      <c r="C70" s="32" t="n"/>
+      <c r="D70" s="33" t="n"/>
       <c r="E70" s="22">
         <f>SUM(E5:E69)</f>
         <v/>
@@ -29448,7 +29485,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -31257,9 +31293,9 @@
           <t>TOTAL HARI INI</t>
         </is>
       </c>
-      <c r="B62" s="21" t="n"/>
-      <c r="C62" s="21" t="n"/>
-      <c r="D62" s="21" t="n"/>
+      <c r="B62" s="32" t="n"/>
+      <c r="C62" s="32" t="n"/>
+      <c r="D62" s="33" t="n"/>
       <c r="E62" s="22">
         <f>SUM(E5:E61)</f>
         <v/>
@@ -31312,7 +31348,6 @@
         </is>
       </c>
     </row>
-    <row r="3"/>
     <row r="4" ht="28" customHeight="1">
       <c r="A4" s="31" t="inlineStr">
         <is>
@@ -32441,9 +32476,9 @@
           <t>TOTAL HARI INI</t>
         </is>
       </c>
-      <c r="B40" s="21" t="n"/>
-      <c r="C40" s="21" t="n"/>
-      <c r="D40" s="21" t="n"/>
+      <c r="B40" s="32" t="n"/>
+      <c r="C40" s="32" t="n"/>
+      <c r="D40" s="33" t="n"/>
       <c r="E40" s="22">
         <f>SUM(E5:E39)</f>
         <v/>

</xml_diff>

<commit_message>
Update susunan bal Blok 01, Blok 02, Blok 03, Blok 04 dan sinkronisasi barcode master
</commit_message>
<xml_diff>
--- a/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
+++ b/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
@@ -18,6 +18,7 @@
     <sheet name="29 Agustus" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="30 Agustus" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="31 Agustus" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="1 September" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -466,7 +467,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H449"/>
+  <dimension ref="A1:H487"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -13724,22 +13725,28 @@
       </c>
       <c r="B426" s="3" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="C426" s="3" t="n">
         <v>601</v>
       </c>
-      <c r="D426" s="3" t="inlineStr"/>
+      <c r="D426" s="3" t="inlineStr">
+        <is>
+          <t>31993</t>
+        </is>
+      </c>
       <c r="E426" s="3" t="inlineStr">
         <is>
-          <t>65</t>
-        </is>
-      </c>
-      <c r="F426" s="3" t="inlineStr"/>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F426" s="3" t="n">
+        <v>50</v>
+      </c>
       <c r="G426" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SELESAI</t>
         </is>
       </c>
       <c r="H426" s="3" t="inlineStr"/>
@@ -13750,22 +13757,28 @@
       </c>
       <c r="B427" s="2" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="C427" s="2" t="n">
         <v>602</v>
       </c>
-      <c r="D427" s="2" t="inlineStr"/>
+      <c r="D427" s="2" t="inlineStr">
+        <is>
+          <t>35339</t>
+        </is>
+      </c>
       <c r="E427" s="2" t="inlineStr">
         <is>
-          <t>65</t>
-        </is>
-      </c>
-      <c r="F427" s="2" t="inlineStr"/>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F427" s="2" t="n">
+        <v>48</v>
+      </c>
       <c r="G427" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SELESAI</t>
         </is>
       </c>
       <c r="H427" s="2" t="inlineStr"/>
@@ -13936,16 +13949,20 @@
       </c>
       <c r="B433" s="2" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="C433" s="2" t="n">
         <v>608</v>
       </c>
-      <c r="D433" s="2" t="inlineStr"/>
+      <c r="D433" s="2" t="inlineStr">
+        <is>
+          <t>35340</t>
+        </is>
+      </c>
       <c r="E433" s="2" t="inlineStr">
         <is>
-          <t>70</t>
+          <t>67</t>
         </is>
       </c>
       <c r="F433" s="2" t="n">
@@ -13953,7 +13970,7 @@
       </c>
       <c r="G433" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SELESAI</t>
         </is>
       </c>
       <c r="H433" s="2" t="inlineStr"/>
@@ -14469,6 +14486,1222 @@
         </is>
       </c>
       <c r="H449" s="2" t="inlineStr"/>
+    </row>
+    <row r="450" ht="20" customHeight="1">
+      <c r="A450" s="3" t="n">
+        <v>446</v>
+      </c>
+      <c r="B450" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C450" s="3" t="n">
+        <v>625</v>
+      </c>
+      <c r="D450" s="3" t="inlineStr">
+        <is>
+          <t>35088</t>
+        </is>
+      </c>
+      <c r="E450" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F450" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="G450" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H450" s="3" t="inlineStr"/>
+    </row>
+    <row r="451" ht="20" customHeight="1">
+      <c r="A451" s="2" t="n">
+        <v>447</v>
+      </c>
+      <c r="B451" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C451" s="2" t="n">
+        <v>626</v>
+      </c>
+      <c r="D451" s="2" t="inlineStr">
+        <is>
+          <t>31989</t>
+        </is>
+      </c>
+      <c r="E451" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F451" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="G451" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H451" s="2" t="inlineStr"/>
+    </row>
+    <row r="452" ht="20" customHeight="1">
+      <c r="A452" s="3" t="n">
+        <v>448</v>
+      </c>
+      <c r="B452" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C452" s="3" t="n">
+        <v>627</v>
+      </c>
+      <c r="D452" s="3" t="inlineStr">
+        <is>
+          <t>31990</t>
+        </is>
+      </c>
+      <c r="E452" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F452" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="G452" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H452" s="3" t="inlineStr"/>
+    </row>
+    <row r="453" ht="20" customHeight="1">
+      <c r="A453" s="2" t="n">
+        <v>449</v>
+      </c>
+      <c r="B453" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C453" s="2" t="n">
+        <v>628</v>
+      </c>
+      <c r="D453" s="2" t="inlineStr">
+        <is>
+          <t>31995</t>
+        </is>
+      </c>
+      <c r="E453" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F453" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G453" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H453" s="2" t="inlineStr"/>
+    </row>
+    <row r="454" ht="20" customHeight="1">
+      <c r="A454" s="3" t="n">
+        <v>450</v>
+      </c>
+      <c r="B454" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C454" s="3" t="n">
+        <v>629</v>
+      </c>
+      <c r="D454" s="3" t="inlineStr">
+        <is>
+          <t>31994</t>
+        </is>
+      </c>
+      <c r="E454" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F454" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="G454" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H454" s="3" t="inlineStr"/>
+    </row>
+    <row r="455" ht="20" customHeight="1">
+      <c r="A455" s="2" t="n">
+        <v>451</v>
+      </c>
+      <c r="B455" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C455" s="2" t="n">
+        <v>630</v>
+      </c>
+      <c r="D455" s="2" t="inlineStr">
+        <is>
+          <t>35082</t>
+        </is>
+      </c>
+      <c r="E455" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F455" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G455" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H455" s="2" t="inlineStr"/>
+    </row>
+    <row r="456" ht="20" customHeight="1">
+      <c r="A456" s="3" t="n">
+        <v>452</v>
+      </c>
+      <c r="B456" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C456" s="3" t="n">
+        <v>631</v>
+      </c>
+      <c r="D456" s="3" t="inlineStr">
+        <is>
+          <t>35087</t>
+        </is>
+      </c>
+      <c r="E456" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F456" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="G456" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H456" s="3" t="inlineStr"/>
+    </row>
+    <row r="457" ht="20" customHeight="1">
+      <c r="A457" s="2" t="n">
+        <v>453</v>
+      </c>
+      <c r="B457" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C457" s="2" t="n">
+        <v>632</v>
+      </c>
+      <c r="D457" s="2" t="inlineStr">
+        <is>
+          <t>35079</t>
+        </is>
+      </c>
+      <c r="E457" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F457" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="G457" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H457" s="2" t="inlineStr"/>
+    </row>
+    <row r="458" ht="20" customHeight="1">
+      <c r="A458" s="3" t="n">
+        <v>454</v>
+      </c>
+      <c r="B458" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C458" s="3" t="n">
+        <v>633</v>
+      </c>
+      <c r="D458" s="3" t="inlineStr">
+        <is>
+          <t>35078</t>
+        </is>
+      </c>
+      <c r="E458" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F458" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="G458" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H458" s="3" t="inlineStr"/>
+    </row>
+    <row r="459" ht="20" customHeight="1">
+      <c r="A459" s="2" t="n">
+        <v>455</v>
+      </c>
+      <c r="B459" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C459" s="2" t="n">
+        <v>634</v>
+      </c>
+      <c r="D459" s="2" t="inlineStr">
+        <is>
+          <t>35080</t>
+        </is>
+      </c>
+      <c r="E459" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F459" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G459" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H459" s="2" t="inlineStr"/>
+    </row>
+    <row r="460" ht="20" customHeight="1">
+      <c r="A460" s="3" t="n">
+        <v>456</v>
+      </c>
+      <c r="B460" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C460" s="3" t="n">
+        <v>635</v>
+      </c>
+      <c r="D460" s="3" t="inlineStr">
+        <is>
+          <t>35663</t>
+        </is>
+      </c>
+      <c r="E460" s="3" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="F460" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="G460" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H460" s="3" t="inlineStr"/>
+    </row>
+    <row r="461" ht="20" customHeight="1">
+      <c r="A461" s="2" t="n">
+        <v>457</v>
+      </c>
+      <c r="B461" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C461" s="2" t="n">
+        <v>636</v>
+      </c>
+      <c r="D461" s="2" t="inlineStr">
+        <is>
+          <t>35661</t>
+        </is>
+      </c>
+      <c r="E461" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="F461" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="G461" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H461" s="2" t="inlineStr"/>
+    </row>
+    <row r="462" ht="20" customHeight="1">
+      <c r="A462" s="3" t="n">
+        <v>458</v>
+      </c>
+      <c r="B462" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C462" s="3" t="n">
+        <v>637</v>
+      </c>
+      <c r="D462" s="3" t="inlineStr">
+        <is>
+          <t>35729</t>
+        </is>
+      </c>
+      <c r="E462" s="3" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="F462" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="G462" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H462" s="3" t="inlineStr"/>
+    </row>
+    <row r="463" ht="20" customHeight="1">
+      <c r="A463" s="2" t="n">
+        <v>459</v>
+      </c>
+      <c r="B463" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C463" s="2" t="n">
+        <v>638</v>
+      </c>
+      <c r="D463" s="2" t="inlineStr">
+        <is>
+          <t>35732</t>
+        </is>
+      </c>
+      <c r="E463" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F463" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="G463" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H463" s="2" t="inlineStr"/>
+    </row>
+    <row r="464" ht="20" customHeight="1">
+      <c r="A464" s="3" t="n">
+        <v>460</v>
+      </c>
+      <c r="B464" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C464" s="3" t="n">
+        <v>639</v>
+      </c>
+      <c r="D464" s="3" t="inlineStr">
+        <is>
+          <t>35731</t>
+        </is>
+      </c>
+      <c r="E464" s="3" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="F464" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="G464" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H464" s="3" t="inlineStr"/>
+    </row>
+    <row r="465" ht="20" customHeight="1">
+      <c r="A465" s="2" t="n">
+        <v>461</v>
+      </c>
+      <c r="B465" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C465" s="2" t="n">
+        <v>640</v>
+      </c>
+      <c r="D465" s="2" t="inlineStr">
+        <is>
+          <t>35730</t>
+        </is>
+      </c>
+      <c r="E465" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="F465" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="G465" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H465" s="2" t="inlineStr"/>
+    </row>
+    <row r="466" ht="20" customHeight="1">
+      <c r="A466" s="3" t="n">
+        <v>462</v>
+      </c>
+      <c r="B466" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C466" s="3" t="n">
+        <v>641</v>
+      </c>
+      <c r="D466" s="3" t="inlineStr">
+        <is>
+          <t>35734</t>
+        </is>
+      </c>
+      <c r="E466" s="3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F466" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="G466" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H466" s="3" t="inlineStr"/>
+    </row>
+    <row r="467" ht="20" customHeight="1">
+      <c r="A467" s="2" t="n">
+        <v>463</v>
+      </c>
+      <c r="B467" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C467" s="2" t="n">
+        <v>642</v>
+      </c>
+      <c r="D467" s="2" t="inlineStr">
+        <is>
+          <t>35662</t>
+        </is>
+      </c>
+      <c r="E467" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F467" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="G467" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H467" s="2" t="inlineStr"/>
+    </row>
+    <row r="468" ht="20" customHeight="1">
+      <c r="A468" s="3" t="n">
+        <v>464</v>
+      </c>
+      <c r="B468" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C468" s="3" t="n">
+        <v>643</v>
+      </c>
+      <c r="D468" s="3" t="inlineStr">
+        <is>
+          <t>35736</t>
+        </is>
+      </c>
+      <c r="E468" s="3" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="F468" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="G468" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H468" s="3" t="inlineStr"/>
+    </row>
+    <row r="469" ht="20" customHeight="1">
+      <c r="A469" s="2" t="n">
+        <v>465</v>
+      </c>
+      <c r="B469" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C469" s="2" t="n">
+        <v>644</v>
+      </c>
+      <c r="D469" s="2" t="inlineStr">
+        <is>
+          <t>35733</t>
+        </is>
+      </c>
+      <c r="E469" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="F469" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="G469" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H469" s="2" t="inlineStr"/>
+    </row>
+    <row r="470" ht="20" customHeight="1">
+      <c r="A470" s="3" t="n">
+        <v>466</v>
+      </c>
+      <c r="B470" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C470" s="3" t="n">
+        <v>645</v>
+      </c>
+      <c r="D470" s="3" t="inlineStr">
+        <is>
+          <t>35735</t>
+        </is>
+      </c>
+      <c r="E470" s="3" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="F470" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="G470" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H470" s="3" t="inlineStr"/>
+    </row>
+    <row r="471" ht="20" customHeight="1">
+      <c r="A471" s="2" t="n">
+        <v>467</v>
+      </c>
+      <c r="B471" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C471" s="2" t="n">
+        <v>646</v>
+      </c>
+      <c r="D471" s="2" t="inlineStr">
+        <is>
+          <t>33860</t>
+        </is>
+      </c>
+      <c r="E471" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="F471" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="G471" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H471" s="2" t="inlineStr"/>
+    </row>
+    <row r="472" ht="20" customHeight="1">
+      <c r="A472" s="3" t="n">
+        <v>468</v>
+      </c>
+      <c r="B472" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C472" s="3" t="n">
+        <v>647</v>
+      </c>
+      <c r="D472" s="3" t="inlineStr">
+        <is>
+          <t>33862</t>
+        </is>
+      </c>
+      <c r="E472" s="3" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="F472" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="G472" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H472" s="3" t="inlineStr"/>
+    </row>
+    <row r="473" ht="20" customHeight="1">
+      <c r="A473" s="2" t="n">
+        <v>469</v>
+      </c>
+      <c r="B473" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C473" s="2" t="n">
+        <v>648</v>
+      </c>
+      <c r="D473" s="2" t="inlineStr">
+        <is>
+          <t>33861</t>
+        </is>
+      </c>
+      <c r="E473" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="F473" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G473" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H473" s="2" t="inlineStr"/>
+    </row>
+    <row r="474" ht="20" customHeight="1">
+      <c r="A474" s="3" t="n">
+        <v>470</v>
+      </c>
+      <c r="B474" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C474" s="3" t="n">
+        <v>649</v>
+      </c>
+      <c r="D474" s="3" t="inlineStr">
+        <is>
+          <t>33863</t>
+        </is>
+      </c>
+      <c r="E474" s="3" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="F474" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="G474" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H474" s="3" t="inlineStr"/>
+    </row>
+    <row r="475" ht="20" customHeight="1">
+      <c r="A475" s="2" t="n">
+        <v>471</v>
+      </c>
+      <c r="B475" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C475" s="2" t="n">
+        <v>650</v>
+      </c>
+      <c r="D475" s="2" t="inlineStr">
+        <is>
+          <t>35739</t>
+        </is>
+      </c>
+      <c r="E475" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F475" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G475" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H475" s="2" t="inlineStr"/>
+    </row>
+    <row r="476" ht="20" customHeight="1">
+      <c r="A476" s="3" t="n">
+        <v>472</v>
+      </c>
+      <c r="B476" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C476" s="3" t="n">
+        <v>651</v>
+      </c>
+      <c r="D476" s="3" t="inlineStr">
+        <is>
+          <t>35738</t>
+        </is>
+      </c>
+      <c r="E476" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F476" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="G476" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H476" s="3" t="inlineStr"/>
+    </row>
+    <row r="477" ht="20" customHeight="1">
+      <c r="A477" s="2" t="n">
+        <v>473</v>
+      </c>
+      <c r="B477" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C477" s="2" t="n">
+        <v>652</v>
+      </c>
+      <c r="D477" s="2" t="inlineStr">
+        <is>
+          <t>35737</t>
+        </is>
+      </c>
+      <c r="E477" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F477" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="G477" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H477" s="2" t="inlineStr"/>
+    </row>
+    <row r="478" ht="20" customHeight="1">
+      <c r="A478" s="3" t="n">
+        <v>474</v>
+      </c>
+      <c r="B478" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C478" s="3" t="n">
+        <v>653</v>
+      </c>
+      <c r="D478" s="3" t="inlineStr">
+        <is>
+          <t>35741</t>
+        </is>
+      </c>
+      <c r="E478" s="3" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="F478" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="G478" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H478" s="3" t="inlineStr"/>
+    </row>
+    <row r="479" ht="20" customHeight="1">
+      <c r="A479" s="2" t="n">
+        <v>475</v>
+      </c>
+      <c r="B479" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C479" s="2" t="n">
+        <v>654</v>
+      </c>
+      <c r="D479" s="2" t="inlineStr">
+        <is>
+          <t>35081</t>
+        </is>
+      </c>
+      <c r="E479" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F479" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G479" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H479" s="2" t="inlineStr"/>
+    </row>
+    <row r="480" ht="20" customHeight="1">
+      <c r="A480" s="3" t="n">
+        <v>476</v>
+      </c>
+      <c r="B480" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C480" s="3" t="n">
+        <v>655</v>
+      </c>
+      <c r="D480" s="3" t="inlineStr">
+        <is>
+          <t>31991</t>
+        </is>
+      </c>
+      <c r="E480" s="3" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F480" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="G480" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H480" s="3" t="inlineStr"/>
+    </row>
+    <row r="481" ht="20" customHeight="1">
+      <c r="A481" s="2" t="n">
+        <v>477</v>
+      </c>
+      <c r="B481" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C481" s="2" t="n">
+        <v>656</v>
+      </c>
+      <c r="D481" s="2" t="inlineStr">
+        <is>
+          <t>31992</t>
+        </is>
+      </c>
+      <c r="E481" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F481" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="G481" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H481" s="2" t="inlineStr"/>
+    </row>
+    <row r="482" ht="20" customHeight="1">
+      <c r="A482" s="3" t="n">
+        <v>478</v>
+      </c>
+      <c r="B482" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C482" s="3" t="n">
+        <v>657</v>
+      </c>
+      <c r="D482" s="3" t="inlineStr">
+        <is>
+          <t>35740</t>
+        </is>
+      </c>
+      <c r="E482" s="3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F482" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="G482" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H482" s="3" t="inlineStr"/>
+    </row>
+    <row r="483" ht="20" customHeight="1">
+      <c r="A483" s="2" t="n">
+        <v>479</v>
+      </c>
+      <c r="B483" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C483" s="2" t="n">
+        <v>658</v>
+      </c>
+      <c r="D483" s="2" t="inlineStr">
+        <is>
+          <t>35083</t>
+        </is>
+      </c>
+      <c r="E483" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F483" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="G483" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H483" s="2" t="inlineStr"/>
+    </row>
+    <row r="484" ht="20" customHeight="1">
+      <c r="A484" s="3" t="n">
+        <v>480</v>
+      </c>
+      <c r="B484" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C484" s="3" t="n">
+        <v>659</v>
+      </c>
+      <c r="D484" s="3" t="inlineStr">
+        <is>
+          <t>35084</t>
+        </is>
+      </c>
+      <c r="E484" s="3" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F484" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="G484" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H484" s="3" t="inlineStr"/>
+    </row>
+    <row r="485" ht="20" customHeight="1">
+      <c r="A485" s="2" t="n">
+        <v>481</v>
+      </c>
+      <c r="B485" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C485" s="2" t="n">
+        <v>660</v>
+      </c>
+      <c r="D485" s="2" t="inlineStr">
+        <is>
+          <t>35086</t>
+        </is>
+      </c>
+      <c r="E485" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F485" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G485" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H485" s="2" t="inlineStr"/>
+    </row>
+    <row r="486" ht="20" customHeight="1">
+      <c r="A486" s="3" t="n">
+        <v>482</v>
+      </c>
+      <c r="B486" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C486" s="3" t="n">
+        <v>661</v>
+      </c>
+      <c r="D486" s="3" t="inlineStr">
+        <is>
+          <t>35085</t>
+        </is>
+      </c>
+      <c r="E486" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F486" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="G486" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H486" s="3" t="inlineStr"/>
+    </row>
+    <row r="487" ht="20" customHeight="1">
+      <c r="A487" s="2" t="n">
+        <v>483</v>
+      </c>
+      <c r="B487" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-01</t>
+        </is>
+      </c>
+      <c r="C487" s="2" t="n">
+        <v>662</v>
+      </c>
+      <c r="D487" s="2" t="inlineStr">
+        <is>
+          <t>35341</t>
+        </is>
+      </c>
+      <c r="E487" s="2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F487" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G487" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H487" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -15665,6 +16898,1176 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>No Gudang</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Nomor Barcode</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Berat (Kg)</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>601</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>31993</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>602</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>35339</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>608</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>35340</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>625</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>35088</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>626</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>31989</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>627</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>31990</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>628</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>31995</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>629</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>31994</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>630</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>35082</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>631</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>35087</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>632</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>35079</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>633</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>35078</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>634</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>35080</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>635</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>35663</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>636</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>35661</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>637</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>35729</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>638</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>35732</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>639</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>35731</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>54</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>640</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>35730</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>641</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>35734</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>642</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>35662</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>643</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>35736</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>644</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>35733</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>645</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>35735</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>646</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>33860</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>647</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>33862</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>648</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>33861</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>649</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>33863</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>650</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>35739</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>651</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>35738</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>652</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>35737</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>653</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>35741</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>654</v>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>35081</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>655</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>31991</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>656</v>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>31992</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>657</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>35740</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>658</v>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>35083</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>659</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>35084</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>660</v>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>35086</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr"/>
+    </row>
+    <row r="44" ht="20" customHeight="1">
+      <c r="A44" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="B44" s="3" t="n">
+        <v>661</v>
+      </c>
+      <c r="C44" s="3" t="inlineStr">
+        <is>
+          <t>35085</t>
+        </is>
+      </c>
+      <c r="D44" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E44" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="F44" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G44" s="3" t="inlineStr"/>
+    </row>
+    <row r="45" ht="20" customHeight="1">
+      <c r="A45" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="B45" s="2" t="n">
+        <v>662</v>
+      </c>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>35341</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
fix(layout): ganti bal 118 menjadi 513 di Blok 11 dan sinkronkan data
</commit_message>
<xml_diff>
--- a/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
+++ b/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
@@ -19,6 +19,7 @@
     <sheet name="30 Agustus" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="31 Agustus" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="1 September" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="2 September" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -467,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H487"/>
+  <dimension ref="A1:H511"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -3061,24 +3062,28 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="C87" s="2" t="n">
         <v>212</v>
       </c>
-      <c r="D87" s="2" t="inlineStr"/>
+      <c r="D87" s="2" t="inlineStr">
+        <is>
+          <t>35429</t>
+        </is>
+      </c>
       <c r="E87" s="2" t="inlineStr">
         <is>
-          <t>64</t>
+          <t>65</t>
         </is>
       </c>
       <c r="F87" s="2" t="n">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="G87" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SELESAI</t>
         </is>
       </c>
       <c r="H87" s="2" t="inlineStr"/>
@@ -3733,24 +3738,28 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="C109" s="2" t="n">
         <v>239</v>
       </c>
-      <c r="D109" s="2" t="inlineStr"/>
+      <c r="D109" s="2" t="inlineStr">
+        <is>
+          <t>35427</t>
+        </is>
+      </c>
       <c r="E109" s="2" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>55</t>
         </is>
       </c>
       <c r="F109" s="2" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="G109" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SELESAI</t>
         </is>
       </c>
       <c r="H109" s="2" t="inlineStr"/>
@@ -3761,24 +3770,28 @@
       </c>
       <c r="B110" s="3" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="C110" s="3" t="n">
         <v>240</v>
       </c>
-      <c r="D110" s="3" t="inlineStr"/>
+      <c r="D110" s="3" t="inlineStr">
+        <is>
+          <t>35426</t>
+        </is>
+      </c>
       <c r="E110" s="3" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>63</t>
         </is>
       </c>
       <c r="F110" s="3" t="n">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G110" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SELESAI</t>
         </is>
       </c>
       <c r="H110" s="3" t="inlineStr"/>
@@ -6569,22 +6582,28 @@
       </c>
       <c r="B200" s="3" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="C200" s="3" t="n">
         <v>362</v>
       </c>
-      <c r="D200" s="3" t="inlineStr"/>
+      <c r="D200" s="3" t="inlineStr">
+        <is>
+          <t>35428</t>
+        </is>
+      </c>
       <c r="E200" s="3" t="inlineStr">
         <is>
-          <t>50</t>
-        </is>
-      </c>
-      <c r="F200" s="3" t="inlineStr"/>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="F200" s="3" t="n">
+        <v>30</v>
+      </c>
       <c r="G200" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SELESAI</t>
         </is>
       </c>
       <c r="H200" s="3" t="inlineStr"/>
@@ -15702,6 +15721,770 @@
         </is>
       </c>
       <c r="H487" s="2" t="inlineStr"/>
+    </row>
+    <row r="488" ht="20" customHeight="1">
+      <c r="A488" s="3" t="n">
+        <v>484</v>
+      </c>
+      <c r="B488" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C488" s="3" t="n">
+        <v>663</v>
+      </c>
+      <c r="D488" s="3" t="inlineStr">
+        <is>
+          <t>35999</t>
+        </is>
+      </c>
+      <c r="E488" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F488" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="G488" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H488" s="3" t="inlineStr"/>
+    </row>
+    <row r="489" ht="20" customHeight="1">
+      <c r="A489" s="2" t="n">
+        <v>485</v>
+      </c>
+      <c r="B489" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C489" s="2" t="n">
+        <v>664</v>
+      </c>
+      <c r="D489" s="2" t="inlineStr">
+        <is>
+          <t>35998</t>
+        </is>
+      </c>
+      <c r="E489" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F489" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="G489" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H489" s="2" t="inlineStr"/>
+    </row>
+    <row r="490" ht="20" customHeight="1">
+      <c r="A490" s="3" t="n">
+        <v>486</v>
+      </c>
+      <c r="B490" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C490" s="3" t="n">
+        <v>665</v>
+      </c>
+      <c r="D490" s="3" t="inlineStr">
+        <is>
+          <t>35775</t>
+        </is>
+      </c>
+      <c r="E490" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F490" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="G490" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H490" s="3" t="inlineStr"/>
+    </row>
+    <row r="491" ht="20" customHeight="1">
+      <c r="A491" s="2" t="n">
+        <v>487</v>
+      </c>
+      <c r="B491" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C491" s="2" t="n">
+        <v>666</v>
+      </c>
+      <c r="D491" s="2" t="inlineStr">
+        <is>
+          <t>35776</t>
+        </is>
+      </c>
+      <c r="E491" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F491" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G491" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H491" s="2" t="inlineStr"/>
+    </row>
+    <row r="492" ht="20" customHeight="1">
+      <c r="A492" s="3" t="n">
+        <v>488</v>
+      </c>
+      <c r="B492" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C492" s="3" t="n">
+        <v>667</v>
+      </c>
+      <c r="D492" s="3" t="inlineStr">
+        <is>
+          <t>35774</t>
+        </is>
+      </c>
+      <c r="E492" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F492" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="G492" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H492" s="3" t="inlineStr"/>
+    </row>
+    <row r="493" ht="20" customHeight="1">
+      <c r="A493" s="2" t="n">
+        <v>489</v>
+      </c>
+      <c r="B493" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C493" s="2" t="n">
+        <v>668</v>
+      </c>
+      <c r="D493" s="2" t="inlineStr">
+        <is>
+          <t>35431</t>
+        </is>
+      </c>
+      <c r="E493" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="F493" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="G493" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H493" s="2" t="inlineStr"/>
+    </row>
+    <row r="494" ht="20" customHeight="1">
+      <c r="A494" s="3" t="n">
+        <v>490</v>
+      </c>
+      <c r="B494" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C494" s="3" t="n">
+        <v>669</v>
+      </c>
+      <c r="D494" s="3" t="inlineStr">
+        <is>
+          <t>35996</t>
+        </is>
+      </c>
+      <c r="E494" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F494" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="G494" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H494" s="3" t="inlineStr"/>
+    </row>
+    <row r="495" ht="20" customHeight="1">
+      <c r="A495" s="2" t="n">
+        <v>491</v>
+      </c>
+      <c r="B495" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C495" s="2" t="n">
+        <v>670</v>
+      </c>
+      <c r="D495" s="2" t="inlineStr">
+        <is>
+          <t>33872</t>
+        </is>
+      </c>
+      <c r="E495" s="2" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="F495" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G495" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H495" s="2" t="inlineStr"/>
+    </row>
+    <row r="496" ht="20" customHeight="1">
+      <c r="A496" s="3" t="n">
+        <v>492</v>
+      </c>
+      <c r="B496" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C496" s="3" t="n">
+        <v>671</v>
+      </c>
+      <c r="D496" s="3" t="inlineStr">
+        <is>
+          <t>35997</t>
+        </is>
+      </c>
+      <c r="E496" s="3" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="F496" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="G496" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H496" s="3" t="inlineStr"/>
+    </row>
+    <row r="497" ht="20" customHeight="1">
+      <c r="A497" s="2" t="n">
+        <v>493</v>
+      </c>
+      <c r="B497" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C497" s="2" t="n">
+        <v>672</v>
+      </c>
+      <c r="D497" s="2" t="inlineStr">
+        <is>
+          <t>35430</t>
+        </is>
+      </c>
+      <c r="E497" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="F497" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G497" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H497" s="2" t="inlineStr"/>
+    </row>
+    <row r="498" ht="20" customHeight="1">
+      <c r="A498" s="3" t="n">
+        <v>494</v>
+      </c>
+      <c r="B498" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C498" s="3" t="n">
+        <v>673</v>
+      </c>
+      <c r="D498" s="3" t="inlineStr">
+        <is>
+          <t>35994</t>
+        </is>
+      </c>
+      <c r="E498" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F498" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="G498" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H498" s="3" t="inlineStr"/>
+    </row>
+    <row r="499" ht="20" customHeight="1">
+      <c r="A499" s="2" t="n">
+        <v>495</v>
+      </c>
+      <c r="B499" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C499" s="2" t="n">
+        <v>674</v>
+      </c>
+      <c r="D499" s="2" t="inlineStr">
+        <is>
+          <t>35995</t>
+        </is>
+      </c>
+      <c r="E499" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F499" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G499" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H499" s="2" t="inlineStr"/>
+    </row>
+    <row r="500" ht="20" customHeight="1">
+      <c r="A500" s="3" t="n">
+        <v>496</v>
+      </c>
+      <c r="B500" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C500" s="3" t="n">
+        <v>675</v>
+      </c>
+      <c r="D500" s="3" t="inlineStr">
+        <is>
+          <t>35375</t>
+        </is>
+      </c>
+      <c r="E500" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F500" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="G500" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H500" s="3" t="inlineStr"/>
+    </row>
+    <row r="501" ht="20" customHeight="1">
+      <c r="A501" s="2" t="n">
+        <v>497</v>
+      </c>
+      <c r="B501" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C501" s="2" t="n">
+        <v>676</v>
+      </c>
+      <c r="D501" s="2" t="inlineStr">
+        <is>
+          <t>34660</t>
+        </is>
+      </c>
+      <c r="E501" s="2" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="F501" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="G501" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H501" s="2" t="inlineStr"/>
+    </row>
+    <row r="502" ht="20" customHeight="1">
+      <c r="A502" s="3" t="n">
+        <v>498</v>
+      </c>
+      <c r="B502" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C502" s="3" t="n">
+        <v>677</v>
+      </c>
+      <c r="D502" s="3" t="inlineStr">
+        <is>
+          <t>39066</t>
+        </is>
+      </c>
+      <c r="E502" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F502" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="G502" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H502" s="3" t="inlineStr"/>
+    </row>
+    <row r="503" ht="20" customHeight="1">
+      <c r="A503" s="2" t="n">
+        <v>499</v>
+      </c>
+      <c r="B503" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C503" s="2" t="n">
+        <v>678</v>
+      </c>
+      <c r="D503" s="2" t="inlineStr">
+        <is>
+          <t>39065</t>
+        </is>
+      </c>
+      <c r="E503" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F503" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G503" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H503" s="2" t="inlineStr"/>
+    </row>
+    <row r="504" ht="20" customHeight="1">
+      <c r="A504" s="3" t="n">
+        <v>500</v>
+      </c>
+      <c r="B504" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C504" s="3" t="n">
+        <v>679</v>
+      </c>
+      <c r="D504" s="3" t="inlineStr">
+        <is>
+          <t>35545</t>
+        </is>
+      </c>
+      <c r="E504" s="3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F504" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="G504" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H504" s="3" t="inlineStr"/>
+    </row>
+    <row r="505" ht="20" customHeight="1">
+      <c r="A505" s="2" t="n">
+        <v>501</v>
+      </c>
+      <c r="B505" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C505" s="2" t="n">
+        <v>680</v>
+      </c>
+      <c r="D505" s="2" t="inlineStr">
+        <is>
+          <t>35546</t>
+        </is>
+      </c>
+      <c r="E505" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F505" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G505" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H505" s="2" t="inlineStr"/>
+    </row>
+    <row r="506" ht="20" customHeight="1">
+      <c r="A506" s="3" t="n">
+        <v>502</v>
+      </c>
+      <c r="B506" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C506" s="3" t="n">
+        <v>681</v>
+      </c>
+      <c r="D506" s="3" t="inlineStr">
+        <is>
+          <t>35219</t>
+        </is>
+      </c>
+      <c r="E506" s="3" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="F506" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="G506" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H506" s="3" t="inlineStr"/>
+    </row>
+    <row r="507" ht="20" customHeight="1">
+      <c r="A507" s="2" t="n">
+        <v>503</v>
+      </c>
+      <c r="B507" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C507" s="2" t="n">
+        <v>682</v>
+      </c>
+      <c r="D507" s="2" t="inlineStr"/>
+      <c r="E507" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F507" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="G507" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H507" s="2" t="inlineStr"/>
+    </row>
+    <row r="508" ht="20" customHeight="1">
+      <c r="A508" s="3" t="n">
+        <v>504</v>
+      </c>
+      <c r="B508" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C508" s="3" t="n">
+        <v>683</v>
+      </c>
+      <c r="D508" s="3" t="inlineStr">
+        <is>
+          <t>35818</t>
+        </is>
+      </c>
+      <c r="E508" s="3" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="F508" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="G508" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H508" s="3" t="inlineStr"/>
+    </row>
+    <row r="509" ht="20" customHeight="1">
+      <c r="A509" s="2" t="n">
+        <v>505</v>
+      </c>
+      <c r="B509" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C509" s="2" t="n">
+        <v>684</v>
+      </c>
+      <c r="D509" s="2" t="inlineStr">
+        <is>
+          <t>35819</t>
+        </is>
+      </c>
+      <c r="E509" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="F509" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="G509" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H509" s="2" t="inlineStr"/>
+    </row>
+    <row r="510" ht="20" customHeight="1">
+      <c r="A510" s="3" t="n">
+        <v>506</v>
+      </c>
+      <c r="B510" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C510" s="3" t="n">
+        <v>685</v>
+      </c>
+      <c r="D510" s="3" t="inlineStr">
+        <is>
+          <t>35992</t>
+        </is>
+      </c>
+      <c r="E510" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F510" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="G510" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H510" s="3" t="inlineStr"/>
+    </row>
+    <row r="511" ht="20" customHeight="1">
+      <c r="A511" s="2" t="n">
+        <v>507</v>
+      </c>
+      <c r="B511" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+      <c r="C511" s="2" t="n">
+        <v>686</v>
+      </c>
+      <c r="D511" s="2" t="inlineStr">
+        <is>
+          <t>35993</t>
+        </is>
+      </c>
+      <c r="E511" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="F511" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G511" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H511" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -18068,6 +18851,821 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>No Gudang</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Nomor Barcode</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Berat (Kg)</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>212</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>35429</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>239</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>35427</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>240</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>35426</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>362</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>35428</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>663</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>35999</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>664</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>35998</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>665</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>35775</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>666</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>35776</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>667</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>35774</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>668</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>35431</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>669</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>35996</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>670</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>33872</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>52</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>671</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>35997</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>672</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>35430</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>65</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>673</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>35994</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>674</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>35995</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>675</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>35375</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>676</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>34660</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>677</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>39066</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>678</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>39065</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>679</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>35545</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>680</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>35546</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>681</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>35219</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>682</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr"/>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>683</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>35818</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>684</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>35819</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>63</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>685</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>35992</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>686</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>35993</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>66</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update susunan bal Blok 11, Blok 12, Blok 13, dan Blok 14
</commit_message>
<xml_diff>
--- a/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
+++ b/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
@@ -25,6 +25,7 @@
     <sheet name="5 September" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="6 September" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="7 September" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="8 September" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -473,7 +474,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H664"/>
+  <dimension ref="A1:H703"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -20605,15 +20606,15 @@
       </c>
       <c r="B641" s="2" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="C641" s="2" t="n">
-        <v>834</v>
+        <v>833</v>
       </c>
       <c r="D641" s="2" t="inlineStr">
         <is>
-          <t>39853</t>
+          <t>124372</t>
         </is>
       </c>
       <c r="E641" s="2" t="inlineStr">
@@ -20622,7 +20623,7 @@
         </is>
       </c>
       <c r="F641" s="2" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="G641" s="2" t="inlineStr">
         <is>
@@ -20641,11 +20642,11 @@
         </is>
       </c>
       <c r="C642" s="3" t="n">
-        <v>835</v>
+        <v>834</v>
       </c>
       <c r="D642" s="3" t="inlineStr">
         <is>
-          <t>39856</t>
+          <t>39853</t>
         </is>
       </c>
       <c r="E642" s="3" t="inlineStr">
@@ -20654,7 +20655,7 @@
         </is>
       </c>
       <c r="F642" s="3" t="n">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="G642" s="3" t="inlineStr">
         <is>
@@ -20673,11 +20674,11 @@
         </is>
       </c>
       <c r="C643" s="2" t="n">
-        <v>836</v>
+        <v>835</v>
       </c>
       <c r="D643" s="2" t="inlineStr">
         <is>
-          <t>39854</t>
+          <t>39856</t>
         </is>
       </c>
       <c r="E643" s="2" t="inlineStr">
@@ -20705,11 +20706,11 @@
         </is>
       </c>
       <c r="C644" s="3" t="n">
-        <v>837</v>
+        <v>836</v>
       </c>
       <c r="D644" s="3" t="inlineStr">
         <is>
-          <t>39855</t>
+          <t>39854</t>
         </is>
       </c>
       <c r="E644" s="3" t="inlineStr">
@@ -20737,20 +20738,20 @@
         </is>
       </c>
       <c r="C645" s="2" t="n">
-        <v>838</v>
+        <v>837</v>
       </c>
       <c r="D645" s="2" t="inlineStr">
         <is>
-          <t>39858</t>
+          <t>39855</t>
         </is>
       </c>
       <c r="E645" s="2" t="inlineStr">
         <is>
-          <t>68</t>
+          <t>72</t>
         </is>
       </c>
       <c r="F645" s="2" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="G645" s="2" t="inlineStr">
         <is>
@@ -20769,11 +20770,11 @@
         </is>
       </c>
       <c r="C646" s="3" t="n">
-        <v>839</v>
+        <v>838</v>
       </c>
       <c r="D646" s="3" t="inlineStr">
         <is>
-          <t>39857</t>
+          <t>39858</t>
         </is>
       </c>
       <c r="E646" s="3" t="inlineStr">
@@ -20782,7 +20783,7 @@
         </is>
       </c>
       <c r="F646" s="3" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="G646" s="3" t="inlineStr">
         <is>
@@ -20801,11 +20802,11 @@
         </is>
       </c>
       <c r="C647" s="2" t="n">
-        <v>840</v>
+        <v>839</v>
       </c>
       <c r="D647" s="2" t="inlineStr">
         <is>
-          <t>39859</t>
+          <t>39857</t>
         </is>
       </c>
       <c r="E647" s="2" t="inlineStr">
@@ -20814,7 +20815,7 @@
         </is>
       </c>
       <c r="F647" s="2" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="G647" s="2" t="inlineStr">
         <is>
@@ -20833,20 +20834,20 @@
         </is>
       </c>
       <c r="C648" s="3" t="n">
-        <v>841</v>
+        <v>840</v>
       </c>
       <c r="D648" s="3" t="inlineStr">
         <is>
-          <t>35113</t>
+          <t>39859</t>
         </is>
       </c>
       <c r="E648" s="3" t="inlineStr">
         <is>
-          <t>55</t>
+          <t>68</t>
         </is>
       </c>
       <c r="F648" s="3" t="n">
-        <v>39</v>
+        <v>49</v>
       </c>
       <c r="G648" s="3" t="inlineStr">
         <is>
@@ -20865,11 +20866,11 @@
         </is>
       </c>
       <c r="C649" s="2" t="n">
-        <v>842</v>
+        <v>841</v>
       </c>
       <c r="D649" s="2" t="inlineStr">
         <is>
-          <t>35112</t>
+          <t>35113</t>
         </is>
       </c>
       <c r="E649" s="2" t="inlineStr">
@@ -20878,7 +20879,7 @@
         </is>
       </c>
       <c r="F649" s="2" t="n">
-        <v>47</v>
+        <v>39</v>
       </c>
       <c r="G649" s="2" t="inlineStr">
         <is>
@@ -20897,16 +20898,16 @@
         </is>
       </c>
       <c r="C650" s="3" t="n">
-        <v>843</v>
+        <v>842</v>
       </c>
       <c r="D650" s="3" t="inlineStr">
         <is>
-          <t>123912</t>
+          <t>35112</t>
         </is>
       </c>
       <c r="E650" s="3" t="inlineStr">
         <is>
-          <t>58</t>
+          <t>55</t>
         </is>
       </c>
       <c r="F650" s="3" t="n">
@@ -20929,11 +20930,11 @@
         </is>
       </c>
       <c r="C651" s="2" t="n">
-        <v>844</v>
+        <v>843</v>
       </c>
       <c r="D651" s="2" t="inlineStr">
         <is>
-          <t>123915</t>
+          <t>123912</t>
         </is>
       </c>
       <c r="E651" s="2" t="inlineStr">
@@ -20942,7 +20943,7 @@
         </is>
       </c>
       <c r="F651" s="2" t="n">
-        <v>44</v>
+        <v>47</v>
       </c>
       <c r="G651" s="2" t="inlineStr">
         <is>
@@ -20961,11 +20962,11 @@
         </is>
       </c>
       <c r="C652" s="3" t="n">
-        <v>845</v>
+        <v>844</v>
       </c>
       <c r="D652" s="3" t="inlineStr">
         <is>
-          <t>123916</t>
+          <t>123915</t>
         </is>
       </c>
       <c r="E652" s="3" t="inlineStr">
@@ -20993,11 +20994,11 @@
         </is>
       </c>
       <c r="C653" s="2" t="n">
-        <v>846</v>
+        <v>845</v>
       </c>
       <c r="D653" s="2" t="inlineStr">
         <is>
-          <t>123914</t>
+          <t>123916</t>
         </is>
       </c>
       <c r="E653" s="2" t="inlineStr">
@@ -21025,11 +21026,11 @@
         </is>
       </c>
       <c r="C654" s="3" t="n">
-        <v>847</v>
+        <v>846</v>
       </c>
       <c r="D654" s="3" t="inlineStr">
         <is>
-          <t>123913</t>
+          <t>123914</t>
         </is>
       </c>
       <c r="E654" s="3" t="inlineStr">
@@ -21038,7 +21039,7 @@
         </is>
       </c>
       <c r="F654" s="3" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="G654" s="3" t="inlineStr">
         <is>
@@ -21057,11 +21058,11 @@
         </is>
       </c>
       <c r="C655" s="2" t="n">
-        <v>848</v>
+        <v>847</v>
       </c>
       <c r="D655" s="2" t="inlineStr">
         <is>
-          <t>123917</t>
+          <t>123913</t>
         </is>
       </c>
       <c r="E655" s="2" t="inlineStr">
@@ -21070,7 +21071,7 @@
         </is>
       </c>
       <c r="F655" s="2" t="n">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="G655" s="2" t="inlineStr">
         <is>
@@ -21089,20 +21090,20 @@
         </is>
       </c>
       <c r="C656" s="3" t="n">
-        <v>849</v>
+        <v>848</v>
       </c>
       <c r="D656" s="3" t="inlineStr">
         <is>
-          <t>123919</t>
+          <t>123917</t>
         </is>
       </c>
       <c r="E656" s="3" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>58</t>
         </is>
       </c>
       <c r="F656" s="3" t="n">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="G656" s="3" t="inlineStr">
         <is>
@@ -21121,11 +21122,11 @@
         </is>
       </c>
       <c r="C657" s="2" t="n">
-        <v>850</v>
+        <v>849</v>
       </c>
       <c r="D657" s="2" t="inlineStr">
         <is>
-          <t>123921</t>
+          <t>123919</t>
         </is>
       </c>
       <c r="E657" s="2" t="inlineStr">
@@ -21134,7 +21135,7 @@
         </is>
       </c>
       <c r="F657" s="2" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="G657" s="2" t="inlineStr">
         <is>
@@ -21153,16 +21154,16 @@
         </is>
       </c>
       <c r="C658" s="3" t="n">
-        <v>851</v>
+        <v>850</v>
       </c>
       <c r="D658" s="3" t="inlineStr">
         <is>
-          <t>123918</t>
+          <t>123921</t>
         </is>
       </c>
       <c r="E658" s="3" t="inlineStr">
         <is>
-          <t>57</t>
+          <t>56</t>
         </is>
       </c>
       <c r="F658" s="3" t="n">
@@ -21185,20 +21186,20 @@
         </is>
       </c>
       <c r="C659" s="2" t="n">
-        <v>852</v>
+        <v>851</v>
       </c>
       <c r="D659" s="2" t="inlineStr">
         <is>
-          <t>123920</t>
+          <t>123918</t>
         </is>
       </c>
       <c r="E659" s="2" t="inlineStr">
         <is>
-          <t>56</t>
+          <t>57</t>
         </is>
       </c>
       <c r="F659" s="2" t="n">
-        <v>40</v>
+        <v>48</v>
       </c>
       <c r="G659" s="2" t="inlineStr">
         <is>
@@ -21217,20 +21218,20 @@
         </is>
       </c>
       <c r="C660" s="3" t="n">
-        <v>853</v>
+        <v>852</v>
       </c>
       <c r="D660" s="3" t="inlineStr">
         <is>
-          <t>35117</t>
+          <t>123920</t>
         </is>
       </c>
       <c r="E660" s="3" t="inlineStr">
         <is>
-          <t>50</t>
+          <t>56</t>
         </is>
       </c>
       <c r="F660" s="3" t="n">
-        <v>30</v>
+        <v>40</v>
       </c>
       <c r="G660" s="3" t="inlineStr">
         <is>
@@ -21249,11 +21250,11 @@
         </is>
       </c>
       <c r="C661" s="2" t="n">
-        <v>854</v>
+        <v>853</v>
       </c>
       <c r="D661" s="2" t="inlineStr">
         <is>
-          <t>35114</t>
+          <t>35117</t>
         </is>
       </c>
       <c r="E661" s="2" t="inlineStr">
@@ -21262,7 +21263,7 @@
         </is>
       </c>
       <c r="F661" s="2" t="n">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="G661" s="2" t="inlineStr">
         <is>
@@ -21281,11 +21282,11 @@
         </is>
       </c>
       <c r="C662" s="3" t="n">
-        <v>855</v>
+        <v>854</v>
       </c>
       <c r="D662" s="3" t="inlineStr">
         <is>
-          <t>35116</t>
+          <t>35114</t>
         </is>
       </c>
       <c r="E662" s="3" t="inlineStr">
@@ -21294,7 +21295,7 @@
         </is>
       </c>
       <c r="F662" s="3" t="n">
-        <v>33</v>
+        <v>37</v>
       </c>
       <c r="G662" s="3" t="inlineStr">
         <is>
@@ -21313,11 +21314,11 @@
         </is>
       </c>
       <c r="C663" s="2" t="n">
-        <v>856</v>
+        <v>855</v>
       </c>
       <c r="D663" s="2" t="inlineStr">
         <is>
-          <t>35115</t>
+          <t>35116</t>
         </is>
       </c>
       <c r="E663" s="2" t="inlineStr">
@@ -21345,27 +21346,1255 @@
         </is>
       </c>
       <c r="C664" s="3" t="n">
+        <v>856</v>
+      </c>
+      <c r="D664" s="3" t="inlineStr">
+        <is>
+          <t>35115</t>
+        </is>
+      </c>
+      <c r="E664" s="3" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="F664" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="G664" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H664" s="3" t="inlineStr"/>
+    </row>
+    <row r="665" ht="20" customHeight="1">
+      <c r="A665" s="2" t="n">
+        <v>661</v>
+      </c>
+      <c r="B665" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-07</t>
+        </is>
+      </c>
+      <c r="C665" s="2" t="n">
         <v>857</v>
       </c>
-      <c r="D664" s="3" t="inlineStr">
+      <c r="D665" s="2" t="inlineStr">
         <is>
           <t>123888</t>
         </is>
       </c>
-      <c r="E664" s="3" t="inlineStr">
+      <c r="E665" s="2" t="inlineStr">
         <is>
           <t>66</t>
         </is>
       </c>
-      <c r="F664" s="3" t="n">
+      <c r="F665" s="2" t="n">
         <v>46</v>
       </c>
-      <c r="G664" s="3" t="inlineStr">
-        <is>
-          <t>SELESAI</t>
-        </is>
-      </c>
-      <c r="H664" s="3" t="inlineStr"/>
+      <c r="G665" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H665" s="2" t="inlineStr"/>
+    </row>
+    <row r="666" ht="20" customHeight="1">
+      <c r="A666" s="3" t="n">
+        <v>662</v>
+      </c>
+      <c r="B666" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C666" s="3" t="n">
+        <v>858</v>
+      </c>
+      <c r="D666" s="3" t="inlineStr">
+        <is>
+          <t>124373</t>
+        </is>
+      </c>
+      <c r="E666" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F666" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="G666" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H666" s="3" t="inlineStr"/>
+    </row>
+    <row r="667" ht="20" customHeight="1">
+      <c r="A667" s="2" t="n">
+        <v>663</v>
+      </c>
+      <c r="B667" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C667" s="2" t="n">
+        <v>859</v>
+      </c>
+      <c r="D667" s="2" t="inlineStr"/>
+      <c r="E667" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F667" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="G667" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H667" s="2" t="inlineStr"/>
+    </row>
+    <row r="668" ht="20" customHeight="1">
+      <c r="A668" s="3" t="n">
+        <v>664</v>
+      </c>
+      <c r="B668" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C668" s="3" t="n">
+        <v>860</v>
+      </c>
+      <c r="D668" s="3" t="inlineStr">
+        <is>
+          <t>124284</t>
+        </is>
+      </c>
+      <c r="E668" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F668" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="G668" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H668" s="3" t="inlineStr"/>
+    </row>
+    <row r="669" ht="20" customHeight="1">
+      <c r="A669" s="2" t="n">
+        <v>665</v>
+      </c>
+      <c r="B669" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C669" s="2" t="n">
+        <v>861</v>
+      </c>
+      <c r="D669" s="2" t="inlineStr">
+        <is>
+          <t>124367</t>
+        </is>
+      </c>
+      <c r="E669" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F669" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G669" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H669" s="2" t="inlineStr"/>
+    </row>
+    <row r="670" ht="20" customHeight="1">
+      <c r="A670" s="3" t="n">
+        <v>666</v>
+      </c>
+      <c r="B670" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C670" s="3" t="n">
+        <v>862</v>
+      </c>
+      <c r="D670" s="3" t="inlineStr">
+        <is>
+          <t>124368</t>
+        </is>
+      </c>
+      <c r="E670" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F670" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="G670" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H670" s="3" t="inlineStr"/>
+    </row>
+    <row r="671" ht="20" customHeight="1">
+      <c r="A671" s="2" t="n">
+        <v>667</v>
+      </c>
+      <c r="B671" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C671" s="2" t="n">
+        <v>863</v>
+      </c>
+      <c r="D671" s="2" t="inlineStr">
+        <is>
+          <t>124370</t>
+        </is>
+      </c>
+      <c r="E671" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F671" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G671" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H671" s="2" t="inlineStr"/>
+    </row>
+    <row r="672" ht="20" customHeight="1">
+      <c r="A672" s="3" t="n">
+        <v>668</v>
+      </c>
+      <c r="B672" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C672" s="3" t="n">
+        <v>864</v>
+      </c>
+      <c r="D672" s="3" t="inlineStr"/>
+      <c r="E672" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F672" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="G672" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H672" s="3" t="inlineStr"/>
+    </row>
+    <row r="673" ht="20" customHeight="1">
+      <c r="A673" s="2" t="n">
+        <v>669</v>
+      </c>
+      <c r="B673" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C673" s="2" t="n">
+        <v>865</v>
+      </c>
+      <c r="D673" s="2" t="inlineStr"/>
+      <c r="E673" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F673" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G673" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H673" s="2" t="inlineStr"/>
+    </row>
+    <row r="674" ht="20" customHeight="1">
+      <c r="A674" s="3" t="n">
+        <v>670</v>
+      </c>
+      <c r="B674" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C674" s="3" t="n">
+        <v>866</v>
+      </c>
+      <c r="D674" s="3" t="inlineStr">
+        <is>
+          <t>124371</t>
+        </is>
+      </c>
+      <c r="E674" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F674" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="G674" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H674" s="3" t="inlineStr"/>
+    </row>
+    <row r="675" ht="20" customHeight="1">
+      <c r="A675" s="2" t="n">
+        <v>671</v>
+      </c>
+      <c r="B675" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C675" s="2" t="n">
+        <v>867</v>
+      </c>
+      <c r="D675" s="2" t="inlineStr"/>
+      <c r="E675" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F675" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G675" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H675" s="2" t="inlineStr"/>
+    </row>
+    <row r="676" ht="20" customHeight="1">
+      <c r="A676" s="3" t="n">
+        <v>672</v>
+      </c>
+      <c r="B676" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C676" s="3" t="n">
+        <v>868</v>
+      </c>
+      <c r="D676" s="3" t="inlineStr">
+        <is>
+          <t>124369</t>
+        </is>
+      </c>
+      <c r="E676" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F676" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="G676" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H676" s="3" t="inlineStr"/>
+    </row>
+    <row r="677" ht="20" customHeight="1">
+      <c r="A677" s="2" t="n">
+        <v>673</v>
+      </c>
+      <c r="B677" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C677" s="2" t="n">
+        <v>869</v>
+      </c>
+      <c r="D677" s="2" t="inlineStr">
+        <is>
+          <t>124285</t>
+        </is>
+      </c>
+      <c r="E677" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F677" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G677" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H677" s="2" t="inlineStr"/>
+    </row>
+    <row r="678" ht="20" customHeight="1">
+      <c r="A678" s="3" t="n">
+        <v>674</v>
+      </c>
+      <c r="B678" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C678" s="3" t="n">
+        <v>870</v>
+      </c>
+      <c r="D678" s="3" t="inlineStr">
+        <is>
+          <t>39833</t>
+        </is>
+      </c>
+      <c r="E678" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F678" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="G678" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H678" s="3" t="inlineStr"/>
+    </row>
+    <row r="679" ht="20" customHeight="1">
+      <c r="A679" s="2" t="n">
+        <v>675</v>
+      </c>
+      <c r="B679" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C679" s="2" t="n">
+        <v>871</v>
+      </c>
+      <c r="D679" s="2" t="inlineStr"/>
+      <c r="E679" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F679" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G679" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H679" s="2" t="inlineStr"/>
+    </row>
+    <row r="680" ht="20" customHeight="1">
+      <c r="A680" s="3" t="n">
+        <v>676</v>
+      </c>
+      <c r="B680" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C680" s="3" t="n">
+        <v>872</v>
+      </c>
+      <c r="D680" s="3" t="inlineStr">
+        <is>
+          <t>124366</t>
+        </is>
+      </c>
+      <c r="E680" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F680" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="G680" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H680" s="3" t="inlineStr"/>
+    </row>
+    <row r="681" ht="20" customHeight="1">
+      <c r="A681" s="2" t="n">
+        <v>677</v>
+      </c>
+      <c r="B681" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C681" s="2" t="n">
+        <v>873</v>
+      </c>
+      <c r="D681" s="2" t="inlineStr">
+        <is>
+          <t>33879</t>
+        </is>
+      </c>
+      <c r="E681" s="2" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="F681" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="G681" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H681" s="2" t="inlineStr"/>
+    </row>
+    <row r="682" ht="20" customHeight="1">
+      <c r="A682" s="3" t="n">
+        <v>678</v>
+      </c>
+      <c r="B682" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C682" s="3" t="n">
+        <v>874</v>
+      </c>
+      <c r="D682" s="3" t="inlineStr">
+        <is>
+          <t>123934</t>
+        </is>
+      </c>
+      <c r="E682" s="3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F682" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="G682" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H682" s="3" t="inlineStr"/>
+    </row>
+    <row r="683" ht="20" customHeight="1">
+      <c r="A683" s="2" t="n">
+        <v>679</v>
+      </c>
+      <c r="B683" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C683" s="2" t="n">
+        <v>875</v>
+      </c>
+      <c r="D683" s="2" t="inlineStr">
+        <is>
+          <t>123935</t>
+        </is>
+      </c>
+      <c r="E683" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="F683" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="G683" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H683" s="2" t="inlineStr"/>
+    </row>
+    <row r="684" ht="20" customHeight="1">
+      <c r="A684" s="3" t="n">
+        <v>680</v>
+      </c>
+      <c r="B684" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C684" s="3" t="n">
+        <v>876</v>
+      </c>
+      <c r="D684" s="3" t="inlineStr">
+        <is>
+          <t>123933</t>
+        </is>
+      </c>
+      <c r="E684" s="3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F684" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="G684" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H684" s="3" t="inlineStr"/>
+    </row>
+    <row r="685" ht="20" customHeight="1">
+      <c r="A685" s="2" t="n">
+        <v>681</v>
+      </c>
+      <c r="B685" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C685" s="2" t="n">
+        <v>877</v>
+      </c>
+      <c r="D685" s="2" t="inlineStr">
+        <is>
+          <t>123944</t>
+        </is>
+      </c>
+      <c r="E685" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F685" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="G685" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H685" s="2" t="inlineStr"/>
+    </row>
+    <row r="686" ht="20" customHeight="1">
+      <c r="A686" s="3" t="n">
+        <v>682</v>
+      </c>
+      <c r="B686" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C686" s="3" t="n">
+        <v>878</v>
+      </c>
+      <c r="D686" s="3" t="inlineStr">
+        <is>
+          <t>123932</t>
+        </is>
+      </c>
+      <c r="E686" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="F686" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="G686" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H686" s="3" t="inlineStr"/>
+    </row>
+    <row r="687" ht="20" customHeight="1">
+      <c r="A687" s="2" t="n">
+        <v>683</v>
+      </c>
+      <c r="B687" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C687" s="2" t="n">
+        <v>879</v>
+      </c>
+      <c r="D687" s="2" t="inlineStr">
+        <is>
+          <t>123929</t>
+        </is>
+      </c>
+      <c r="E687" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="F687" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="G687" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H687" s="2" t="inlineStr"/>
+    </row>
+    <row r="688" ht="20" customHeight="1">
+      <c r="A688" s="3" t="n">
+        <v>684</v>
+      </c>
+      <c r="B688" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C688" s="3" t="n">
+        <v>880</v>
+      </c>
+      <c r="D688" s="3" t="inlineStr">
+        <is>
+          <t>123931</t>
+        </is>
+      </c>
+      <c r="E688" s="3" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="F688" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="G688" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H688" s="3" t="inlineStr"/>
+    </row>
+    <row r="689" ht="20" customHeight="1">
+      <c r="A689" s="2" t="n">
+        <v>685</v>
+      </c>
+      <c r="B689" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C689" s="2" t="n">
+        <v>881</v>
+      </c>
+      <c r="D689" s="2" t="inlineStr">
+        <is>
+          <t>123930</t>
+        </is>
+      </c>
+      <c r="E689" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="F689" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="G689" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H689" s="2" t="inlineStr"/>
+    </row>
+    <row r="690" ht="20" customHeight="1">
+      <c r="A690" s="3" t="n">
+        <v>686</v>
+      </c>
+      <c r="B690" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C690" s="3" t="n">
+        <v>882</v>
+      </c>
+      <c r="D690" s="3" t="inlineStr">
+        <is>
+          <t>123941</t>
+        </is>
+      </c>
+      <c r="E690" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F690" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="G690" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H690" s="3" t="inlineStr"/>
+    </row>
+    <row r="691" ht="20" customHeight="1">
+      <c r="A691" s="2" t="n">
+        <v>687</v>
+      </c>
+      <c r="B691" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C691" s="2" t="n">
+        <v>883</v>
+      </c>
+      <c r="D691" s="2" t="inlineStr">
+        <is>
+          <t>124227</t>
+        </is>
+      </c>
+      <c r="E691" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F691" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G691" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H691" s="2" t="inlineStr"/>
+    </row>
+    <row r="692" ht="20" customHeight="1">
+      <c r="A692" s="3" t="n">
+        <v>688</v>
+      </c>
+      <c r="B692" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C692" s="3" t="n">
+        <v>884</v>
+      </c>
+      <c r="D692" s="3" t="inlineStr">
+        <is>
+          <t>123940</t>
+        </is>
+      </c>
+      <c r="E692" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F692" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="G692" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H692" s="3" t="inlineStr"/>
+    </row>
+    <row r="693" ht="20" customHeight="1">
+      <c r="A693" s="2" t="n">
+        <v>689</v>
+      </c>
+      <c r="B693" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C693" s="2" t="n">
+        <v>885</v>
+      </c>
+      <c r="D693" s="2" t="inlineStr">
+        <is>
+          <t>123943</t>
+        </is>
+      </c>
+      <c r="E693" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F693" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="G693" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H693" s="2" t="inlineStr"/>
+    </row>
+    <row r="694" ht="20" customHeight="1">
+      <c r="A694" s="3" t="n">
+        <v>690</v>
+      </c>
+      <c r="B694" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C694" s="3" t="n">
+        <v>886</v>
+      </c>
+      <c r="D694" s="3" t="inlineStr">
+        <is>
+          <t>123942</t>
+        </is>
+      </c>
+      <c r="E694" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F694" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="G694" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H694" s="3" t="inlineStr"/>
+    </row>
+    <row r="695" ht="20" customHeight="1">
+      <c r="A695" s="2" t="n">
+        <v>691</v>
+      </c>
+      <c r="B695" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C695" s="2" t="n">
+        <v>887</v>
+      </c>
+      <c r="D695" s="2" t="inlineStr">
+        <is>
+          <t>123937</t>
+        </is>
+      </c>
+      <c r="E695" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="F695" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="G695" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H695" s="2" t="inlineStr"/>
+    </row>
+    <row r="696" ht="20" customHeight="1">
+      <c r="A696" s="3" t="n">
+        <v>692</v>
+      </c>
+      <c r="B696" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C696" s="3" t="n">
+        <v>888</v>
+      </c>
+      <c r="D696" s="3" t="inlineStr">
+        <is>
+          <t>33883</t>
+        </is>
+      </c>
+      <c r="E696" s="3" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="F696" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="G696" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H696" s="3" t="inlineStr"/>
+    </row>
+    <row r="697" ht="20" customHeight="1">
+      <c r="A697" s="2" t="n">
+        <v>693</v>
+      </c>
+      <c r="B697" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C697" s="2" t="n">
+        <v>889</v>
+      </c>
+      <c r="D697" s="2" t="inlineStr">
+        <is>
+          <t>123936</t>
+        </is>
+      </c>
+      <c r="E697" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="F697" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="G697" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H697" s="2" t="inlineStr"/>
+    </row>
+    <row r="698" ht="20" customHeight="1">
+      <c r="A698" s="3" t="n">
+        <v>694</v>
+      </c>
+      <c r="B698" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C698" s="3" t="n">
+        <v>890</v>
+      </c>
+      <c r="D698" s="3" t="inlineStr">
+        <is>
+          <t>123938</t>
+        </is>
+      </c>
+      <c r="E698" s="3" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="F698" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="G698" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H698" s="3" t="inlineStr"/>
+    </row>
+    <row r="699" ht="20" customHeight="1">
+      <c r="A699" s="2" t="n">
+        <v>695</v>
+      </c>
+      <c r="B699" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C699" s="2" t="n">
+        <v>891</v>
+      </c>
+      <c r="D699" s="2" t="inlineStr">
+        <is>
+          <t>123939</t>
+        </is>
+      </c>
+      <c r="E699" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="F699" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="G699" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H699" s="2" t="inlineStr"/>
+    </row>
+    <row r="700" ht="20" customHeight="1">
+      <c r="A700" s="3" t="n">
+        <v>696</v>
+      </c>
+      <c r="B700" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C700" s="3" t="n">
+        <v>892</v>
+      </c>
+      <c r="D700" s="3" t="inlineStr">
+        <is>
+          <t>33881</t>
+        </is>
+      </c>
+      <c r="E700" s="3" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="F700" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="G700" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H700" s="3" t="inlineStr"/>
+    </row>
+    <row r="701" ht="20" customHeight="1">
+      <c r="A701" s="2" t="n">
+        <v>697</v>
+      </c>
+      <c r="B701" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C701" s="2" t="n">
+        <v>893</v>
+      </c>
+      <c r="D701" s="2" t="inlineStr">
+        <is>
+          <t>33884</t>
+        </is>
+      </c>
+      <c r="E701" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="F701" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="G701" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H701" s="2" t="inlineStr"/>
+    </row>
+    <row r="702" ht="20" customHeight="1">
+      <c r="A702" s="3" t="n">
+        <v>698</v>
+      </c>
+      <c r="B702" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C702" s="3" t="n">
+        <v>894</v>
+      </c>
+      <c r="D702" s="3" t="inlineStr">
+        <is>
+          <t>33880</t>
+        </is>
+      </c>
+      <c r="E702" s="3" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="F702" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="G702" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H702" s="3" t="inlineStr"/>
+    </row>
+    <row r="703" ht="20" customHeight="1">
+      <c r="A703" s="2" t="n">
+        <v>699</v>
+      </c>
+      <c r="B703" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-08</t>
+        </is>
+      </c>
+      <c r="C703" s="2" t="n">
+        <v>895</v>
+      </c>
+      <c r="D703" s="2" t="inlineStr">
+        <is>
+          <t>33882</t>
+        </is>
+      </c>
+      <c r="E703" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="F703" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="G703" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H703" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -28996,6 +30225,1102 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G43"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>No Gudang</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Nomor Barcode</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Berat (Kg)</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>833</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>124372</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>858</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>124373</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>859</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr"/>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>860</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>124284</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>861</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>124367</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>862</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>124368</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>863</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>124370</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>864</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr"/>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>865</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr"/>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>866</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>124371</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>867</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr"/>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>868</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>124369</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>869</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>124285</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>870</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>39833</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>871</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>872</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>124366</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>873</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>33879</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>53</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>874</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>123934</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>875</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>123935</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>876</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>123933</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>877</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>123944</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>878</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>123932</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>879</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>123929</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>880</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>123931</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>881</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>123930</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr"/>
+    </row>
+    <row r="30" ht="20" customHeight="1">
+      <c r="A30" s="3" t="n">
+        <v>26</v>
+      </c>
+      <c r="B30" s="3" t="n">
+        <v>882</v>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>123941</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31" ht="20" customHeight="1">
+      <c r="A31" s="2" t="n">
+        <v>27</v>
+      </c>
+      <c r="B31" s="2" t="n">
+        <v>883</v>
+      </c>
+      <c r="C31" s="2" t="inlineStr">
+        <is>
+          <t>124227</t>
+        </is>
+      </c>
+      <c r="D31" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E31" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F31" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G31" s="2" t="inlineStr"/>
+    </row>
+    <row r="32" ht="20" customHeight="1">
+      <c r="A32" s="3" t="n">
+        <v>28</v>
+      </c>
+      <c r="B32" s="3" t="n">
+        <v>884</v>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>123940</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr"/>
+    </row>
+    <row r="33" ht="20" customHeight="1">
+      <c r="A33" s="2" t="n">
+        <v>29</v>
+      </c>
+      <c r="B33" s="2" t="n">
+        <v>885</v>
+      </c>
+      <c r="C33" s="2" t="inlineStr">
+        <is>
+          <t>123943</t>
+        </is>
+      </c>
+      <c r="D33" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E33" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="F33" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G33" s="2" t="inlineStr"/>
+    </row>
+    <row r="34" ht="20" customHeight="1">
+      <c r="A34" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="B34" s="3" t="n">
+        <v>886</v>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>123942</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr"/>
+    </row>
+    <row r="35" ht="20" customHeight="1">
+      <c r="A35" s="2" t="n">
+        <v>31</v>
+      </c>
+      <c r="B35" s="2" t="n">
+        <v>887</v>
+      </c>
+      <c r="C35" s="2" t="inlineStr">
+        <is>
+          <t>123937</t>
+        </is>
+      </c>
+      <c r="D35" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E35" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="F35" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G35" s="2" t="inlineStr"/>
+    </row>
+    <row r="36" ht="20" customHeight="1">
+      <c r="A36" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="B36" s="3" t="n">
+        <v>888</v>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>33883</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="n">
+        <v>50</v>
+      </c>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37" ht="20" customHeight="1">
+      <c r="A37" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="B37" s="2" t="n">
+        <v>889</v>
+      </c>
+      <c r="C37" s="2" t="inlineStr">
+        <is>
+          <t>123936</t>
+        </is>
+      </c>
+      <c r="D37" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E37" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="F37" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G37" s="2" t="inlineStr"/>
+    </row>
+    <row r="38" ht="20" customHeight="1">
+      <c r="A38" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="B38" s="3" t="n">
+        <v>890</v>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>123938</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39" ht="20" customHeight="1">
+      <c r="A39" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="B39" s="2" t="n">
+        <v>891</v>
+      </c>
+      <c r="C39" s="2" t="inlineStr">
+        <is>
+          <t>123939</t>
+        </is>
+      </c>
+      <c r="D39" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E39" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="F39" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G39" s="2" t="inlineStr"/>
+    </row>
+    <row r="40" ht="20" customHeight="1">
+      <c r="A40" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="B40" s="3" t="n">
+        <v>892</v>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>33881</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="n">
+        <v>34</v>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr"/>
+    </row>
+    <row r="41" ht="20" customHeight="1">
+      <c r="A41" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="B41" s="2" t="n">
+        <v>893</v>
+      </c>
+      <c r="C41" s="2" t="inlineStr">
+        <is>
+          <t>33884</t>
+        </is>
+      </c>
+      <c r="D41" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E41" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="F41" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G41" s="2" t="inlineStr"/>
+    </row>
+    <row r="42" ht="20" customHeight="1">
+      <c r="A42" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="B42" s="3" t="n">
+        <v>894</v>
+      </c>
+      <c r="C42" s="3" t="inlineStr">
+        <is>
+          <t>33880</t>
+        </is>
+      </c>
+      <c r="D42" s="3" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E42" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="F42" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G42" s="3" t="inlineStr"/>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="B43" s="2" t="n">
+        <v>895</v>
+      </c>
+      <c r="C43" s="2" t="inlineStr">
+        <is>
+          <t>33882</t>
+        </is>
+      </c>
+      <c r="D43" s="2" t="inlineStr">
+        <is>
+          <t>50</t>
+        </is>
+      </c>
+      <c r="E43" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="F43" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G43" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update susunan bal Blok 01, Blok 02, Blok 03, Blok 07, Blok 08, Blok 10 dan update script/laporan
</commit_message>
<xml_diff>
--- a/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
+++ b/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
@@ -26,6 +26,8 @@
     <sheet name="6 September" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="7 September" sheetId="18" state="visible" r:id="rId18"/>
     <sheet name="8 September" sheetId="19" state="visible" r:id="rId19"/>
+    <sheet name="9 September" sheetId="20" state="visible" r:id="rId20"/>
+    <sheet name="10 September" sheetId="21" state="visible" r:id="rId21"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -474,7 +476,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H703"/>
+  <dimension ref="A1:H740"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -21438,13 +21440,17 @@
       </c>
       <c r="B667" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="C667" s="2" t="n">
         <v>859</v>
       </c>
-      <c r="D667" s="2" t="inlineStr"/>
+      <c r="D667" s="2" t="inlineStr">
+        <is>
+          <t>124853</t>
+        </is>
+      </c>
       <c r="E667" s="2" t="inlineStr">
         <is>
           <t>72</t>
@@ -21455,7 +21461,7 @@
       </c>
       <c r="G667" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SELESAI</t>
         </is>
       </c>
       <c r="H667" s="2" t="inlineStr"/>
@@ -21594,13 +21600,17 @@
       </c>
       <c r="B672" s="3" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="C672" s="3" t="n">
         <v>864</v>
       </c>
-      <c r="D672" s="3" t="inlineStr"/>
+      <c r="D672" s="3" t="inlineStr">
+        <is>
+          <t>124851</t>
+        </is>
+      </c>
       <c r="E672" s="3" t="inlineStr">
         <is>
           <t>72</t>
@@ -21611,7 +21621,7 @@
       </c>
       <c r="G672" s="3" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SELESAI</t>
         </is>
       </c>
       <c r="H672" s="3" t="inlineStr"/>
@@ -21622,13 +21632,17 @@
       </c>
       <c r="B673" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="C673" s="2" t="n">
         <v>865</v>
       </c>
-      <c r="D673" s="2" t="inlineStr"/>
+      <c r="D673" s="2" t="inlineStr">
+        <is>
+          <t>124852</t>
+        </is>
+      </c>
       <c r="E673" s="2" t="inlineStr">
         <is>
           <t>72</t>
@@ -21639,7 +21653,7 @@
       </c>
       <c r="G673" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SELESAI</t>
         </is>
       </c>
       <c r="H673" s="2" t="inlineStr"/>
@@ -21682,13 +21696,17 @@
       </c>
       <c r="B675" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="C675" s="2" t="n">
         <v>867</v>
       </c>
-      <c r="D675" s="2" t="inlineStr"/>
+      <c r="D675" s="2" t="inlineStr">
+        <is>
+          <t>124586</t>
+        </is>
+      </c>
       <c r="E675" s="2" t="inlineStr">
         <is>
           <t>72</t>
@@ -21699,7 +21717,7 @@
       </c>
       <c r="G675" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SELESAI</t>
         </is>
       </c>
       <c r="H675" s="2" t="inlineStr"/>
@@ -21806,13 +21824,17 @@
       </c>
       <c r="B679" s="2" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="C679" s="2" t="n">
         <v>871</v>
       </c>
-      <c r="D679" s="2" t="inlineStr"/>
+      <c r="D679" s="2" t="inlineStr">
+        <is>
+          <t>124250</t>
+        </is>
+      </c>
       <c r="E679" s="2" t="inlineStr">
         <is>
           <t>72</t>
@@ -21823,7 +21845,7 @@
       </c>
       <c r="G679" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>SELESAI</t>
         </is>
       </c>
       <c r="H679" s="2" t="inlineStr"/>
@@ -22595,6 +22617,1182 @@
         </is>
       </c>
       <c r="H703" s="2" t="inlineStr"/>
+    </row>
+    <row r="704" ht="20" customHeight="1">
+      <c r="A704" s="3" t="n">
+        <v>700</v>
+      </c>
+      <c r="B704" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C704" s="3" t="n">
+        <v>899</v>
+      </c>
+      <c r="D704" s="3" t="inlineStr">
+        <is>
+          <t>124854</t>
+        </is>
+      </c>
+      <c r="E704" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F704" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="G704" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H704" s="3" t="inlineStr"/>
+    </row>
+    <row r="705" ht="20" customHeight="1">
+      <c r="A705" s="2" t="n">
+        <v>701</v>
+      </c>
+      <c r="B705" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C705" s="2" t="n">
+        <v>900</v>
+      </c>
+      <c r="D705" s="2" t="inlineStr">
+        <is>
+          <t>124855</t>
+        </is>
+      </c>
+      <c r="E705" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F705" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="G705" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H705" s="2" t="inlineStr"/>
+    </row>
+    <row r="706" ht="20" customHeight="1">
+      <c r="A706" s="3" t="n">
+        <v>702</v>
+      </c>
+      <c r="B706" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C706" s="3" t="n">
+        <v>901</v>
+      </c>
+      <c r="D706" s="3" t="inlineStr">
+        <is>
+          <t>124856</t>
+        </is>
+      </c>
+      <c r="E706" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F706" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="G706" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H706" s="3" t="inlineStr"/>
+    </row>
+    <row r="707" ht="20" customHeight="1">
+      <c r="A707" s="2" t="n">
+        <v>703</v>
+      </c>
+      <c r="B707" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C707" s="2" t="n">
+        <v>902</v>
+      </c>
+      <c r="D707" s="2" t="inlineStr">
+        <is>
+          <t>124857</t>
+        </is>
+      </c>
+      <c r="E707" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F707" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="G707" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H707" s="2" t="inlineStr"/>
+    </row>
+    <row r="708" ht="20" customHeight="1">
+      <c r="A708" s="3" t="n">
+        <v>704</v>
+      </c>
+      <c r="B708" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C708" s="3" t="n">
+        <v>903</v>
+      </c>
+      <c r="D708" s="3" t="inlineStr">
+        <is>
+          <t>124526</t>
+        </is>
+      </c>
+      <c r="E708" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="F708" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="G708" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H708" s="3" t="inlineStr"/>
+    </row>
+    <row r="709" ht="20" customHeight="1">
+      <c r="A709" s="2" t="n">
+        <v>705</v>
+      </c>
+      <c r="B709" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C709" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="D709" s="2" t="inlineStr">
+        <is>
+          <t>124588</t>
+        </is>
+      </c>
+      <c r="E709" s="2" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="F709" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="G709" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H709" s="2" t="inlineStr"/>
+    </row>
+    <row r="710" ht="20" customHeight="1">
+      <c r="A710" s="3" t="n">
+        <v>706</v>
+      </c>
+      <c r="B710" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C710" s="3" t="n">
+        <v>905</v>
+      </c>
+      <c r="D710" s="3" t="inlineStr">
+        <is>
+          <t>124587</t>
+        </is>
+      </c>
+      <c r="E710" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F710" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="G710" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H710" s="3" t="inlineStr"/>
+    </row>
+    <row r="711" ht="20" customHeight="1">
+      <c r="A711" s="2" t="n">
+        <v>707</v>
+      </c>
+      <c r="B711" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C711" s="2" t="n">
+        <v>907</v>
+      </c>
+      <c r="D711" s="2" t="inlineStr">
+        <is>
+          <t>33889</t>
+        </is>
+      </c>
+      <c r="E711" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="F711" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="G711" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H711" s="2" t="inlineStr"/>
+    </row>
+    <row r="712" ht="20" customHeight="1">
+      <c r="A712" s="3" t="n">
+        <v>708</v>
+      </c>
+      <c r="B712" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C712" s="3" t="n">
+        <v>911</v>
+      </c>
+      <c r="D712" s="3" t="inlineStr">
+        <is>
+          <t>124808</t>
+        </is>
+      </c>
+      <c r="E712" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F712" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="G712" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H712" s="3" t="inlineStr"/>
+    </row>
+    <row r="713" ht="20" customHeight="1">
+      <c r="A713" s="2" t="n">
+        <v>709</v>
+      </c>
+      <c r="B713" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C713" s="2" t="n">
+        <v>912</v>
+      </c>
+      <c r="D713" s="2" t="inlineStr">
+        <is>
+          <t>124589</t>
+        </is>
+      </c>
+      <c r="E713" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F713" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G713" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H713" s="2" t="inlineStr"/>
+    </row>
+    <row r="714" ht="20" customHeight="1">
+      <c r="A714" s="3" t="n">
+        <v>710</v>
+      </c>
+      <c r="B714" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C714" s="3" t="n">
+        <v>913</v>
+      </c>
+      <c r="D714" s="3" t="inlineStr">
+        <is>
+          <t>33890</t>
+        </is>
+      </c>
+      <c r="E714" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="F714" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="G714" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H714" s="3" t="inlineStr"/>
+    </row>
+    <row r="715" ht="20" customHeight="1">
+      <c r="A715" s="2" t="n">
+        <v>711</v>
+      </c>
+      <c r="B715" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C715" s="2" t="n">
+        <v>914</v>
+      </c>
+      <c r="D715" s="2" t="inlineStr">
+        <is>
+          <t>124525</t>
+        </is>
+      </c>
+      <c r="E715" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="F715" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="G715" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H715" s="2" t="inlineStr"/>
+    </row>
+    <row r="716" ht="20" customHeight="1">
+      <c r="A716" s="3" t="n">
+        <v>712</v>
+      </c>
+      <c r="B716" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C716" s="3" t="n">
+        <v>915</v>
+      </c>
+      <c r="D716" s="3" t="inlineStr">
+        <is>
+          <t>124523</t>
+        </is>
+      </c>
+      <c r="E716" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="F716" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="G716" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H716" s="3" t="inlineStr"/>
+    </row>
+    <row r="717" ht="20" customHeight="1">
+      <c r="A717" s="2" t="n">
+        <v>713</v>
+      </c>
+      <c r="B717" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-09</t>
+        </is>
+      </c>
+      <c r="C717" s="2" t="n">
+        <v>916</v>
+      </c>
+      <c r="D717" s="2" t="inlineStr">
+        <is>
+          <t>124524</t>
+        </is>
+      </c>
+      <c r="E717" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="F717" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="G717" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H717" s="2" t="inlineStr"/>
+    </row>
+    <row r="718" ht="20" customHeight="1">
+      <c r="A718" s="3" t="n">
+        <v>714</v>
+      </c>
+      <c r="B718" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C718" s="3" t="n">
+        <v>917</v>
+      </c>
+      <c r="D718" s="3" t="inlineStr">
+        <is>
+          <t>125244</t>
+        </is>
+      </c>
+      <c r="E718" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F718" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="G718" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H718" s="3" t="inlineStr"/>
+    </row>
+    <row r="719" ht="20" customHeight="1">
+      <c r="A719" s="2" t="n">
+        <v>715</v>
+      </c>
+      <c r="B719" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C719" s="2" t="n">
+        <v>918</v>
+      </c>
+      <c r="D719" s="2" t="inlineStr">
+        <is>
+          <t>125245</t>
+        </is>
+      </c>
+      <c r="E719" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F719" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="G719" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H719" s="2" t="inlineStr"/>
+    </row>
+    <row r="720" ht="20" customHeight="1">
+      <c r="A720" s="3" t="n">
+        <v>716</v>
+      </c>
+      <c r="B720" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C720" s="3" t="n">
+        <v>919</v>
+      </c>
+      <c r="D720" s="3" t="inlineStr">
+        <is>
+          <t>125057</t>
+        </is>
+      </c>
+      <c r="E720" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F720" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="G720" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H720" s="3" t="inlineStr"/>
+    </row>
+    <row r="721" ht="20" customHeight="1">
+      <c r="A721" s="2" t="n">
+        <v>717</v>
+      </c>
+      <c r="B721" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C721" s="2" t="n">
+        <v>920</v>
+      </c>
+      <c r="D721" s="2" t="inlineStr">
+        <is>
+          <t>125055</t>
+        </is>
+      </c>
+      <c r="E721" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F721" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="G721" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H721" s="2" t="inlineStr"/>
+    </row>
+    <row r="722" ht="20" customHeight="1">
+      <c r="A722" s="3" t="n">
+        <v>718</v>
+      </c>
+      <c r="B722" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C722" s="3" t="n">
+        <v>921</v>
+      </c>
+      <c r="D722" s="3" t="inlineStr">
+        <is>
+          <t>125242</t>
+        </is>
+      </c>
+      <c r="E722" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F722" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="G722" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H722" s="3" t="inlineStr"/>
+    </row>
+    <row r="723" ht="20" customHeight="1">
+      <c r="A723" s="2" t="n">
+        <v>719</v>
+      </c>
+      <c r="B723" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C723" s="2" t="n">
+        <v>922</v>
+      </c>
+      <c r="D723" s="2" t="inlineStr">
+        <is>
+          <t>125243</t>
+        </is>
+      </c>
+      <c r="E723" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F723" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="G723" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H723" s="2" t="inlineStr"/>
+    </row>
+    <row r="724" ht="20" customHeight="1">
+      <c r="A724" s="3" t="n">
+        <v>720</v>
+      </c>
+      <c r="B724" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C724" s="3" t="n">
+        <v>923</v>
+      </c>
+      <c r="D724" s="3" t="inlineStr">
+        <is>
+          <t>125058</t>
+        </is>
+      </c>
+      <c r="E724" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F724" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="G724" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H724" s="3" t="inlineStr"/>
+    </row>
+    <row r="725" ht="20" customHeight="1">
+      <c r="A725" s="2" t="n">
+        <v>721</v>
+      </c>
+      <c r="B725" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C725" s="2" t="n">
+        <v>924</v>
+      </c>
+      <c r="D725" s="2" t="inlineStr">
+        <is>
+          <t>125056</t>
+        </is>
+      </c>
+      <c r="E725" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F725" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="G725" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H725" s="2" t="inlineStr"/>
+    </row>
+    <row r="726" ht="20" customHeight="1">
+      <c r="A726" s="3" t="n">
+        <v>722</v>
+      </c>
+      <c r="B726" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C726" s="3" t="n">
+        <v>925</v>
+      </c>
+      <c r="D726" s="3" t="inlineStr">
+        <is>
+          <t>125059</t>
+        </is>
+      </c>
+      <c r="E726" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F726" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="G726" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H726" s="3" t="inlineStr"/>
+    </row>
+    <row r="727" ht="20" customHeight="1">
+      <c r="A727" s="2" t="n">
+        <v>723</v>
+      </c>
+      <c r="B727" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C727" s="2" t="n">
+        <v>926</v>
+      </c>
+      <c r="D727" s="2" t="inlineStr">
+        <is>
+          <t>125246</t>
+        </is>
+      </c>
+      <c r="E727" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F727" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="G727" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H727" s="2" t="inlineStr"/>
+    </row>
+    <row r="728" ht="20" customHeight="1">
+      <c r="A728" s="3" t="n">
+        <v>724</v>
+      </c>
+      <c r="B728" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C728" s="3" t="n">
+        <v>927</v>
+      </c>
+      <c r="D728" s="3" t="inlineStr">
+        <is>
+          <t>125061</t>
+        </is>
+      </c>
+      <c r="E728" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F728" s="3" t="n">
+        <v>35</v>
+      </c>
+      <c r="G728" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H728" s="3" t="inlineStr"/>
+    </row>
+    <row r="729" ht="20" customHeight="1">
+      <c r="A729" s="2" t="n">
+        <v>725</v>
+      </c>
+      <c r="B729" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C729" s="2" t="n">
+        <v>928</v>
+      </c>
+      <c r="D729" s="2" t="inlineStr">
+        <is>
+          <t>125247</t>
+        </is>
+      </c>
+      <c r="E729" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F729" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="G729" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H729" s="2" t="inlineStr"/>
+    </row>
+    <row r="730" ht="20" customHeight="1">
+      <c r="A730" s="3" t="n">
+        <v>726</v>
+      </c>
+      <c r="B730" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C730" s="3" t="n">
+        <v>929</v>
+      </c>
+      <c r="D730" s="3" t="inlineStr">
+        <is>
+          <t>125248</t>
+        </is>
+      </c>
+      <c r="E730" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F730" s="3" t="n">
+        <v>32</v>
+      </c>
+      <c r="G730" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H730" s="3" t="inlineStr"/>
+    </row>
+    <row r="731" ht="20" customHeight="1">
+      <c r="A731" s="2" t="n">
+        <v>727</v>
+      </c>
+      <c r="B731" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C731" s="2" t="n">
+        <v>930</v>
+      </c>
+      <c r="D731" s="2" t="inlineStr"/>
+      <c r="E731" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F731" s="2" t="n">
+        <v>39</v>
+      </c>
+      <c r="G731" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H731" s="2" t="inlineStr"/>
+    </row>
+    <row r="732" ht="20" customHeight="1">
+      <c r="A732" s="3" t="n">
+        <v>728</v>
+      </c>
+      <c r="B732" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C732" s="3" t="n">
+        <v>931</v>
+      </c>
+      <c r="D732" s="3" t="inlineStr"/>
+      <c r="E732" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F732" s="3" t="n">
+        <v>30</v>
+      </c>
+      <c r="G732" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="H732" s="3" t="inlineStr"/>
+    </row>
+    <row r="733" ht="20" customHeight="1">
+      <c r="A733" s="2" t="n">
+        <v>729</v>
+      </c>
+      <c r="B733" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C733" s="2" t="n">
+        <v>932</v>
+      </c>
+      <c r="D733" s="2" t="inlineStr">
+        <is>
+          <t>125060</t>
+        </is>
+      </c>
+      <c r="E733" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F733" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="G733" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H733" s="2" t="inlineStr"/>
+    </row>
+    <row r="734" ht="20" customHeight="1">
+      <c r="A734" s="3" t="n">
+        <v>730</v>
+      </c>
+      <c r="B734" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C734" s="3" t="n">
+        <v>933</v>
+      </c>
+      <c r="D734" s="3" t="inlineStr">
+        <is>
+          <t>125062</t>
+        </is>
+      </c>
+      <c r="E734" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F734" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="G734" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H734" s="3" t="inlineStr"/>
+    </row>
+    <row r="735" ht="20" customHeight="1">
+      <c r="A735" s="2" t="n">
+        <v>731</v>
+      </c>
+      <c r="B735" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C735" s="2" t="n">
+        <v>934</v>
+      </c>
+      <c r="D735" s="2" t="inlineStr">
+        <is>
+          <t>124539</t>
+        </is>
+      </c>
+      <c r="E735" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F735" s="2" t="n">
+        <v>49</v>
+      </c>
+      <c r="G735" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H735" s="2" t="inlineStr"/>
+    </row>
+    <row r="736" ht="20" customHeight="1">
+      <c r="A736" s="3" t="n">
+        <v>732</v>
+      </c>
+      <c r="B736" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C736" s="3" t="n">
+        <v>935</v>
+      </c>
+      <c r="D736" s="3" t="inlineStr">
+        <is>
+          <t>124538</t>
+        </is>
+      </c>
+      <c r="E736" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F736" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="G736" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H736" s="3" t="inlineStr"/>
+    </row>
+    <row r="737" ht="20" customHeight="1">
+      <c r="A737" s="2" t="n">
+        <v>733</v>
+      </c>
+      <c r="B737" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C737" s="2" t="n">
+        <v>936</v>
+      </c>
+      <c r="D737" s="2" t="inlineStr">
+        <is>
+          <t>124537</t>
+        </is>
+      </c>
+      <c r="E737" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F737" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="G737" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H737" s="2" t="inlineStr"/>
+    </row>
+    <row r="738" ht="20" customHeight="1">
+      <c r="A738" s="3" t="n">
+        <v>734</v>
+      </c>
+      <c r="B738" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C738" s="3" t="n">
+        <v>937</v>
+      </c>
+      <c r="D738" s="3" t="inlineStr">
+        <is>
+          <t>124536</t>
+        </is>
+      </c>
+      <c r="E738" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="F738" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="G738" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H738" s="3" t="inlineStr"/>
+    </row>
+    <row r="739" ht="20" customHeight="1">
+      <c r="A739" s="2" t="n">
+        <v>735</v>
+      </c>
+      <c r="B739" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C739" s="2" t="n">
+        <v>938</v>
+      </c>
+      <c r="D739" s="2" t="inlineStr">
+        <is>
+          <t>125053</t>
+        </is>
+      </c>
+      <c r="E739" s="2" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="F739" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="G739" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H739" s="2" t="inlineStr"/>
+    </row>
+    <row r="740" ht="20" customHeight="1">
+      <c r="A740" s="3" t="n">
+        <v>736</v>
+      </c>
+      <c r="B740" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="C740" s="3" t="n">
+        <v>939</v>
+      </c>
+      <c r="D740" s="3" t="inlineStr">
+        <is>
+          <t>125054</t>
+        </is>
+      </c>
+      <c r="E740" s="3" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="F740" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="G740" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H740" s="3" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -33013,6 +34211,1258 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet20.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>No Gudang</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Nomor Barcode</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Berat (Kg)</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>859</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>124853</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>864</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>124851</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>865</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>124852</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>867</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>124586</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>871</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>124250</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>50</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>899</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>124854</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>900</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>124855</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>901</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>124856</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>38</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>902</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>124857</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>903</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>124526</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>904</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>124588</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>43</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>905</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>124587</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>907</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>33889</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>911</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>124808</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>912</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>124589</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>913</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>33890</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>914</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>124525</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>915</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>124523</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>916</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>124524</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet21.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G27"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>No Gudang</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Nomor Barcode</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Berat (Kg)</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>917</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>125244</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>918</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>125245</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>919</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>125057</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>920</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>125055</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>921</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>125242</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>40</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>922</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>125243</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>923</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>125058</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>44</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>924</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>125056</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>925</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>125059</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>42</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>926</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>125246</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>44</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>927</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>125061</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>35</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>928</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>125247</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>929</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>125248</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>32</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>930</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr"/>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>931</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>932</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>125060</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>36</v>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>933</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>125062</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>38</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>934</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>124539</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>935</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>124538</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>936</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>124537</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>33</v>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>937</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>124536</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>56</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>36</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>938</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>125053</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>43</v>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>939</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>125054</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>71</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update susunan bal Blok 01, Blok 02, Blok 03 (tambah dari atas) dan sinkronisasi laporan/web
</commit_message>
<xml_diff>
--- a/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
+++ b/Dokumen_Rekap_NoGud_Barkot_Kg.xlsx
@@ -28,6 +28,7 @@
     <sheet name="8 September" sheetId="19" state="visible" r:id="rId19"/>
     <sheet name="9 September" sheetId="20" state="visible" r:id="rId20"/>
     <sheet name="10 September" sheetId="21" state="visible" r:id="rId21"/>
+    <sheet name="11 September" sheetId="22" state="visible" r:id="rId22"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -476,7 +477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H740"/>
+  <dimension ref="A1:H765"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -23793,6 +23794,806 @@
         </is>
       </c>
       <c r="H740" s="3" t="inlineStr"/>
+    </row>
+    <row r="741" ht="20" customHeight="1">
+      <c r="A741" s="2" t="n">
+        <v>737</v>
+      </c>
+      <c r="B741" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C741" s="2" t="n">
+        <v>940</v>
+      </c>
+      <c r="D741" s="2" t="inlineStr">
+        <is>
+          <t>125295</t>
+        </is>
+      </c>
+      <c r="E741" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F741" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="G741" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H741" s="2" t="inlineStr"/>
+    </row>
+    <row r="742" ht="20" customHeight="1">
+      <c r="A742" s="3" t="n">
+        <v>738</v>
+      </c>
+      <c r="B742" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C742" s="3" t="n">
+        <v>941</v>
+      </c>
+      <c r="D742" s="3" t="inlineStr">
+        <is>
+          <t>125291</t>
+        </is>
+      </c>
+      <c r="E742" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F742" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="G742" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H742" s="3" t="inlineStr"/>
+    </row>
+    <row r="743" ht="20" customHeight="1">
+      <c r="A743" s="2" t="n">
+        <v>739</v>
+      </c>
+      <c r="B743" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C743" s="2" t="n">
+        <v>942</v>
+      </c>
+      <c r="D743" s="2" t="inlineStr">
+        <is>
+          <t>125292</t>
+        </is>
+      </c>
+      <c r="E743" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F743" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G743" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H743" s="2" t="inlineStr"/>
+    </row>
+    <row r="744" ht="20" customHeight="1">
+      <c r="A744" s="3" t="n">
+        <v>740</v>
+      </c>
+      <c r="B744" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C744" s="3" t="n">
+        <v>943</v>
+      </c>
+      <c r="D744" s="3" t="inlineStr">
+        <is>
+          <t>125293</t>
+        </is>
+      </c>
+      <c r="E744" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F744" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="G744" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H744" s="3" t="inlineStr"/>
+    </row>
+    <row r="745" ht="20" customHeight="1">
+      <c r="A745" s="2" t="n">
+        <v>741</v>
+      </c>
+      <c r="B745" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C745" s="2" t="n">
+        <v>944</v>
+      </c>
+      <c r="D745" s="2" t="inlineStr">
+        <is>
+          <t>125294</t>
+        </is>
+      </c>
+      <c r="E745" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F745" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="G745" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H745" s="2" t="inlineStr"/>
+    </row>
+    <row r="746" ht="20" customHeight="1">
+      <c r="A746" s="3" t="n">
+        <v>742</v>
+      </c>
+      <c r="B746" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C746" s="3" t="n">
+        <v>945</v>
+      </c>
+      <c r="D746" s="3" t="inlineStr">
+        <is>
+          <t>125581</t>
+        </is>
+      </c>
+      <c r="E746" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F746" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="G746" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H746" s="3" t="inlineStr"/>
+    </row>
+    <row r="747" ht="20" customHeight="1">
+      <c r="A747" s="2" t="n">
+        <v>743</v>
+      </c>
+      <c r="B747" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C747" s="2" t="n">
+        <v>946</v>
+      </c>
+      <c r="D747" s="2" t="inlineStr">
+        <is>
+          <t>125582</t>
+        </is>
+      </c>
+      <c r="E747" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F747" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="G747" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H747" s="2" t="inlineStr"/>
+    </row>
+    <row r="748" ht="20" customHeight="1">
+      <c r="A748" s="3" t="n">
+        <v>744</v>
+      </c>
+      <c r="B748" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C748" s="3" t="n">
+        <v>947</v>
+      </c>
+      <c r="D748" s="3" t="inlineStr">
+        <is>
+          <t>125479</t>
+        </is>
+      </c>
+      <c r="E748" s="3" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="F748" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="G748" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H748" s="3" t="inlineStr"/>
+    </row>
+    <row r="749" ht="20" customHeight="1">
+      <c r="A749" s="2" t="n">
+        <v>745</v>
+      </c>
+      <c r="B749" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C749" s="2" t="n">
+        <v>948</v>
+      </c>
+      <c r="D749" s="2" t="inlineStr">
+        <is>
+          <t>125480</t>
+        </is>
+      </c>
+      <c r="E749" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="F749" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="G749" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H749" s="2" t="inlineStr"/>
+    </row>
+    <row r="750" ht="20" customHeight="1">
+      <c r="A750" s="3" t="n">
+        <v>746</v>
+      </c>
+      <c r="B750" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C750" s="3" t="n">
+        <v>949</v>
+      </c>
+      <c r="D750" s="3" t="inlineStr">
+        <is>
+          <t>125481</t>
+        </is>
+      </c>
+      <c r="E750" s="3" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="F750" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="G750" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H750" s="3" t="inlineStr"/>
+    </row>
+    <row r="751" ht="20" customHeight="1">
+      <c r="A751" s="2" t="n">
+        <v>747</v>
+      </c>
+      <c r="B751" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C751" s="2" t="n">
+        <v>950</v>
+      </c>
+      <c r="D751" s="2" t="inlineStr">
+        <is>
+          <t>125482</t>
+        </is>
+      </c>
+      <c r="E751" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="F751" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="G751" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H751" s="2" t="inlineStr"/>
+    </row>
+    <row r="752" ht="20" customHeight="1">
+      <c r="A752" s="3" t="n">
+        <v>748</v>
+      </c>
+      <c r="B752" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C752" s="3" t="n">
+        <v>951</v>
+      </c>
+      <c r="D752" s="3" t="inlineStr">
+        <is>
+          <t>124544</t>
+        </is>
+      </c>
+      <c r="E752" s="3" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="F752" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="G752" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H752" s="3" t="inlineStr"/>
+    </row>
+    <row r="753" ht="20" customHeight="1">
+      <c r="A753" s="2" t="n">
+        <v>749</v>
+      </c>
+      <c r="B753" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C753" s="2" t="n">
+        <v>952</v>
+      </c>
+      <c r="D753" s="2" t="inlineStr">
+        <is>
+          <t>124545</t>
+        </is>
+      </c>
+      <c r="E753" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="F753" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="G753" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H753" s="2" t="inlineStr"/>
+    </row>
+    <row r="754" ht="20" customHeight="1">
+      <c r="A754" s="3" t="n">
+        <v>750</v>
+      </c>
+      <c r="B754" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C754" s="3" t="n">
+        <v>953</v>
+      </c>
+      <c r="D754" s="3" t="inlineStr">
+        <is>
+          <t>125334</t>
+        </is>
+      </c>
+      <c r="E754" s="3" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="F754" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="G754" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H754" s="3" t="inlineStr"/>
+    </row>
+    <row r="755" ht="20" customHeight="1">
+      <c r="A755" s="2" t="n">
+        <v>751</v>
+      </c>
+      <c r="B755" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C755" s="2" t="n">
+        <v>954</v>
+      </c>
+      <c r="D755" s="2" t="inlineStr">
+        <is>
+          <t>125296</t>
+        </is>
+      </c>
+      <c r="E755" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F755" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="G755" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H755" s="2" t="inlineStr"/>
+    </row>
+    <row r="756" ht="20" customHeight="1">
+      <c r="A756" s="3" t="n">
+        <v>752</v>
+      </c>
+      <c r="B756" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C756" s="3" t="n">
+        <v>955</v>
+      </c>
+      <c r="D756" s="3" t="inlineStr">
+        <is>
+          <t>125297</t>
+        </is>
+      </c>
+      <c r="E756" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="F756" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="G756" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H756" s="3" t="inlineStr"/>
+    </row>
+    <row r="757" ht="20" customHeight="1">
+      <c r="A757" s="2" t="n">
+        <v>753</v>
+      </c>
+      <c r="B757" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C757" s="2" t="n">
+        <v>956</v>
+      </c>
+      <c r="D757" s="2" t="inlineStr">
+        <is>
+          <t>124546</t>
+        </is>
+      </c>
+      <c r="E757" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="F757" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="G757" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H757" s="2" t="inlineStr"/>
+    </row>
+    <row r="758" ht="20" customHeight="1">
+      <c r="A758" s="3" t="n">
+        <v>754</v>
+      </c>
+      <c r="B758" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C758" s="3" t="n">
+        <v>957</v>
+      </c>
+      <c r="D758" s="3" t="inlineStr">
+        <is>
+          <t>35121</t>
+        </is>
+      </c>
+      <c r="E758" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="F758" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="G758" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H758" s="3" t="inlineStr"/>
+    </row>
+    <row r="759" ht="20" customHeight="1">
+      <c r="A759" s="2" t="n">
+        <v>755</v>
+      </c>
+      <c r="B759" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C759" s="2" t="n">
+        <v>958</v>
+      </c>
+      <c r="D759" s="2" t="inlineStr">
+        <is>
+          <t>35120</t>
+        </is>
+      </c>
+      <c r="E759" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="F759" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="G759" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H759" s="2" t="inlineStr"/>
+    </row>
+    <row r="760" ht="20" customHeight="1">
+      <c r="A760" s="3" t="n">
+        <v>756</v>
+      </c>
+      <c r="B760" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C760" s="3" t="n">
+        <v>959</v>
+      </c>
+      <c r="D760" s="3" t="inlineStr">
+        <is>
+          <t>124547</t>
+        </is>
+      </c>
+      <c r="E760" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="F760" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="G760" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H760" s="3" t="inlineStr"/>
+    </row>
+    <row r="761" ht="20" customHeight="1">
+      <c r="A761" s="2" t="n">
+        <v>757</v>
+      </c>
+      <c r="B761" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C761" s="2" t="n">
+        <v>960</v>
+      </c>
+      <c r="D761" s="2" t="inlineStr">
+        <is>
+          <t>35119</t>
+        </is>
+      </c>
+      <c r="E761" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="F761" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="G761" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H761" s="2" t="inlineStr"/>
+    </row>
+    <row r="762" ht="20" customHeight="1">
+      <c r="A762" s="3" t="n">
+        <v>758</v>
+      </c>
+      <c r="B762" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C762" s="3" t="n">
+        <v>961</v>
+      </c>
+      <c r="D762" s="3" t="inlineStr">
+        <is>
+          <t>125475</t>
+        </is>
+      </c>
+      <c r="E762" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F762" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="G762" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H762" s="3" t="inlineStr"/>
+    </row>
+    <row r="763" ht="20" customHeight="1">
+      <c r="A763" s="2" t="n">
+        <v>759</v>
+      </c>
+      <c r="B763" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C763" s="2" t="n">
+        <v>962</v>
+      </c>
+      <c r="D763" s="2" t="inlineStr">
+        <is>
+          <t>125478</t>
+        </is>
+      </c>
+      <c r="E763" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="F763" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="G763" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H763" s="2" t="inlineStr"/>
+    </row>
+    <row r="764" ht="20" customHeight="1">
+      <c r="A764" s="3" t="n">
+        <v>760</v>
+      </c>
+      <c r="B764" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C764" s="3" t="n">
+        <v>963</v>
+      </c>
+      <c r="D764" s="3" t="inlineStr">
+        <is>
+          <t>125476</t>
+        </is>
+      </c>
+      <c r="E764" s="3" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F764" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="G764" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H764" s="3" t="inlineStr"/>
+    </row>
+    <row r="765" ht="20" customHeight="1">
+      <c r="A765" s="2" t="n">
+        <v>761</v>
+      </c>
+      <c r="B765" s="2" t="inlineStr">
+        <is>
+          <t>2026-09-11</t>
+        </is>
+      </c>
+      <c r="C765" s="2" t="n">
+        <v>964</v>
+      </c>
+      <c r="D765" s="2" t="inlineStr">
+        <is>
+          <t>125477</t>
+        </is>
+      </c>
+      <c r="E765" s="2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="F765" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="G765" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="H765" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -35463,6 +36264,744 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet22.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="15" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="15" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1"/>
+    <row r="2"/>
+    <row r="3"/>
+    <row r="4" ht="24" customHeight="1">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="B4" s="1" t="inlineStr">
+        <is>
+          <t>No Gudang</t>
+        </is>
+      </c>
+      <c r="C4" s="1" t="inlineStr">
+        <is>
+          <t>Nomor Barcode</t>
+        </is>
+      </c>
+      <c r="D4" s="1" t="inlineStr">
+        <is>
+          <t>Grade</t>
+        </is>
+      </c>
+      <c r="E4" s="1" t="inlineStr">
+        <is>
+          <t>Berat (Kg)</t>
+        </is>
+      </c>
+      <c r="F4" s="1" t="inlineStr">
+        <is>
+          <t>Status</t>
+        </is>
+      </c>
+      <c r="G4" s="1" t="inlineStr">
+        <is>
+          <t>Keterangan</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="B5" s="2" t="n">
+        <v>940</v>
+      </c>
+      <c r="C5" s="2" t="inlineStr">
+        <is>
+          <t>125295</t>
+        </is>
+      </c>
+      <c r="D5" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E5" s="2" t="n">
+        <v>48</v>
+      </c>
+      <c r="F5" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G5" s="2" t="inlineStr"/>
+    </row>
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="3" t="n">
+        <v>2</v>
+      </c>
+      <c r="B6" s="3" t="n">
+        <v>941</v>
+      </c>
+      <c r="C6" s="3" t="inlineStr">
+        <is>
+          <t>125291</t>
+        </is>
+      </c>
+      <c r="D6" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E6" s="3" t="n">
+        <v>47</v>
+      </c>
+      <c r="F6" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G6" s="3" t="inlineStr"/>
+    </row>
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="B7" s="2" t="n">
+        <v>942</v>
+      </c>
+      <c r="C7" s="2" t="inlineStr">
+        <is>
+          <t>125292</t>
+        </is>
+      </c>
+      <c r="D7" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E7" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="F7" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G7" s="2" t="inlineStr"/>
+    </row>
+    <row r="8" ht="20" customHeight="1">
+      <c r="A8" s="3" t="n">
+        <v>4</v>
+      </c>
+      <c r="B8" s="3" t="n">
+        <v>943</v>
+      </c>
+      <c r="C8" s="3" t="inlineStr">
+        <is>
+          <t>125293</t>
+        </is>
+      </c>
+      <c r="D8" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E8" s="3" t="n">
+        <v>40</v>
+      </c>
+      <c r="F8" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G8" s="3" t="inlineStr"/>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="B9" s="2" t="n">
+        <v>944</v>
+      </c>
+      <c r="C9" s="2" t="inlineStr">
+        <is>
+          <t>125294</t>
+        </is>
+      </c>
+      <c r="D9" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E9" s="2" t="n">
+        <v>45</v>
+      </c>
+      <c r="F9" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G9" s="2" t="inlineStr"/>
+    </row>
+    <row r="10" ht="20" customHeight="1">
+      <c r="A10" s="3" t="n">
+        <v>6</v>
+      </c>
+      <c r="B10" s="3" t="n">
+        <v>945</v>
+      </c>
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>125581</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="F10" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G10" s="3" t="inlineStr"/>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="B11" s="2" t="n">
+        <v>946</v>
+      </c>
+      <c r="C11" s="2" t="inlineStr">
+        <is>
+          <t>125582</t>
+        </is>
+      </c>
+      <c r="D11" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E11" s="2" t="n">
+        <v>33</v>
+      </c>
+      <c r="F11" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G11" s="2" t="inlineStr"/>
+    </row>
+    <row r="12" ht="20" customHeight="1">
+      <c r="A12" s="3" t="n">
+        <v>8</v>
+      </c>
+      <c r="B12" s="3" t="n">
+        <v>947</v>
+      </c>
+      <c r="C12" s="3" t="inlineStr">
+        <is>
+          <t>125479</t>
+        </is>
+      </c>
+      <c r="D12" s="3" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="E12" s="3" t="n">
+        <v>45</v>
+      </c>
+      <c r="F12" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G12" s="3" t="inlineStr"/>
+    </row>
+    <row r="13" ht="20" customHeight="1">
+      <c r="A13" s="2" t="n">
+        <v>9</v>
+      </c>
+      <c r="B13" s="2" t="n">
+        <v>948</v>
+      </c>
+      <c r="C13" s="2" t="inlineStr">
+        <is>
+          <t>125480</t>
+        </is>
+      </c>
+      <c r="D13" s="2" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="E13" s="2" t="n">
+        <v>41</v>
+      </c>
+      <c r="F13" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G13" s="2" t="inlineStr"/>
+    </row>
+    <row r="14" ht="20" customHeight="1">
+      <c r="A14" s="3" t="n">
+        <v>10</v>
+      </c>
+      <c r="B14" s="3" t="n">
+        <v>949</v>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>125481</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>62</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="n">
+        <v>42</v>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="A15" s="2" t="n">
+        <v>11</v>
+      </c>
+      <c r="B15" s="2" t="n">
+        <v>950</v>
+      </c>
+      <c r="C15" s="2" t="inlineStr">
+        <is>
+          <t>125482</t>
+        </is>
+      </c>
+      <c r="D15" s="2" t="inlineStr">
+        <is>
+          <t>70</t>
+        </is>
+      </c>
+      <c r="E15" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="F15" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G15" s="2" t="inlineStr"/>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="A16" s="3" t="n">
+        <v>12</v>
+      </c>
+      <c r="B16" s="3" t="n">
+        <v>951</v>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>124544</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="n">
+        <v>48</v>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr"/>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="A17" s="2" t="n">
+        <v>13</v>
+      </c>
+      <c r="B17" s="2" t="n">
+        <v>952</v>
+      </c>
+      <c r="C17" s="2" t="inlineStr">
+        <is>
+          <t>124545</t>
+        </is>
+      </c>
+      <c r="D17" s="2" t="inlineStr">
+        <is>
+          <t>55</t>
+        </is>
+      </c>
+      <c r="E17" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="F17" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G17" s="2" t="inlineStr"/>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="A18" s="3" t="n">
+        <v>14</v>
+      </c>
+      <c r="B18" s="3" t="n">
+        <v>953</v>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>125334</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>64</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="n">
+        <v>31</v>
+      </c>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="A19" s="2" t="n">
+        <v>15</v>
+      </c>
+      <c r="B19" s="2" t="n">
+        <v>954</v>
+      </c>
+      <c r="C19" s="2" t="inlineStr">
+        <is>
+          <t>125296</t>
+        </is>
+      </c>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="F19" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G19" s="2" t="inlineStr"/>
+    </row>
+    <row r="20" ht="20" customHeight="1">
+      <c r="A20" s="3" t="n">
+        <v>16</v>
+      </c>
+      <c r="B20" s="3" t="n">
+        <v>955</v>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>125297</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>72</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="n">
+        <v>41</v>
+      </c>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21" ht="20" customHeight="1">
+      <c r="A21" s="2" t="n">
+        <v>17</v>
+      </c>
+      <c r="B21" s="2" t="n">
+        <v>956</v>
+      </c>
+      <c r="C21" s="2" t="inlineStr">
+        <is>
+          <t>124546</t>
+        </is>
+      </c>
+      <c r="D21" s="2" t="inlineStr">
+        <is>
+          <t>57</t>
+        </is>
+      </c>
+      <c r="E21" s="2" t="n">
+        <v>46</v>
+      </c>
+      <c r="F21" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G21" s="2" t="inlineStr"/>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="A22" s="3" t="n">
+        <v>18</v>
+      </c>
+      <c r="B22" s="3" t="n">
+        <v>957</v>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>35121</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="n">
+        <v>46</v>
+      </c>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr"/>
+    </row>
+    <row r="23" ht="20" customHeight="1">
+      <c r="A23" s="2" t="n">
+        <v>19</v>
+      </c>
+      <c r="B23" s="2" t="n">
+        <v>958</v>
+      </c>
+      <c r="C23" s="2" t="inlineStr">
+        <is>
+          <t>35120</t>
+        </is>
+      </c>
+      <c r="D23" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E23" s="2" t="n">
+        <v>37</v>
+      </c>
+      <c r="F23" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G23" s="2" t="inlineStr"/>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="A24" s="3" t="n">
+        <v>20</v>
+      </c>
+      <c r="B24" s="3" t="n">
+        <v>959</v>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>124547</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>60</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="n">
+        <v>37</v>
+      </c>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25" ht="20" customHeight="1">
+      <c r="A25" s="2" t="n">
+        <v>21</v>
+      </c>
+      <c r="B25" s="2" t="n">
+        <v>960</v>
+      </c>
+      <c r="C25" s="2" t="inlineStr">
+        <is>
+          <t>35119</t>
+        </is>
+      </c>
+      <c r="D25" s="2" t="inlineStr">
+        <is>
+          <t>58</t>
+        </is>
+      </c>
+      <c r="E25" s="2" t="n">
+        <v>34</v>
+      </c>
+      <c r="F25" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G25" s="2" t="inlineStr"/>
+    </row>
+    <row r="26" ht="20" customHeight="1">
+      <c r="A26" s="3" t="n">
+        <v>22</v>
+      </c>
+      <c r="B26" s="3" t="n">
+        <v>961</v>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>125475</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="n">
+        <v>39</v>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27" ht="20" customHeight="1">
+      <c r="A27" s="2" t="n">
+        <v>23</v>
+      </c>
+      <c r="B27" s="2" t="n">
+        <v>962</v>
+      </c>
+      <c r="C27" s="2" t="inlineStr">
+        <is>
+          <t>125478</t>
+        </is>
+      </c>
+      <c r="D27" s="2" t="inlineStr">
+        <is>
+          <t>68</t>
+        </is>
+      </c>
+      <c r="E27" s="2" t="n">
+        <v>30</v>
+      </c>
+      <c r="F27" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G27" s="2" t="inlineStr"/>
+    </row>
+    <row r="28" ht="20" customHeight="1">
+      <c r="A28" s="3" t="n">
+        <v>24</v>
+      </c>
+      <c r="B28" s="3" t="n">
+        <v>963</v>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>125476</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="n">
+        <v>49</v>
+      </c>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29" ht="20" customHeight="1">
+      <c r="A29" s="2" t="n">
+        <v>25</v>
+      </c>
+      <c r="B29" s="2" t="n">
+        <v>964</v>
+      </c>
+      <c r="C29" s="2" t="inlineStr">
+        <is>
+          <t>125477</t>
+        </is>
+      </c>
+      <c r="D29" s="2" t="inlineStr">
+        <is>
+          <t>67</t>
+        </is>
+      </c>
+      <c r="E29" s="2" t="n">
+        <v>47</v>
+      </c>
+      <c r="F29" s="2" t="inlineStr">
+        <is>
+          <t>SELESAI</t>
+        </is>
+      </c>
+      <c r="G29" s="2" t="inlineStr"/>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>